<commit_message>
Correction des extractions comptables - résultat 2023 = -786,03 €
- Inclusion du compte 6221 (honoraires travaux haie 120€) dans les charges 2023
- Inclusion du compte 6710 (travaux VMC 792€) dans les charges 2024
- Vérification croisée avec les comptes 4711/4721
- Résultats corrigés : 2023=-786€, 2024=+7391€, 2025=+8116€ (partiel)

Co-authored-by: alainannickbaptiste-dot <alainannickbaptiste-dot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/bilan_comptable_comparatif.xlsx
+++ b/bilan_comptable_comparatif.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet name="Bilan Comparatif" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Compte de Résultat" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Détail Bilan par Compte" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,11 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
-    <numFmt numFmtId="165" formatCode=""/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,6 +65,14 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <i val="1"/>
       <color rgb="00FF0000"/>
       <sz val="9"/>
@@ -140,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -183,30 +189,26 @@
     <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -575,7 +577,7 @@
   <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -603,20 +605,17 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2023
-(31/12/2023)</t>
+          <t>31/12/2023</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2024
-(31/12/2024)</t>
+          <t>31/12/2024</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2025
-(20/07/2025)*</t>
+          <t>20/07/2025*</t>
         </is>
       </c>
     </row>
@@ -675,7 +674,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Copropriétaires - soldes débiteurs (450)</t>
+          <t xml:space="preserve">   Fournisseurs - soldes débiteurs (4010)</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
@@ -685,13 +684,13 @@
         <v>0</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>3776.31</v>
+        <v>278.48</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Fournisseurs - soldes débiteurs (4010)</t>
+          <t xml:space="preserve">   Copropriétaires - soldes débiteurs (450)</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
@@ -701,7 +700,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>278.48</v>
+        <v>3776.31</v>
       </c>
     </row>
     <row r="12">
@@ -850,20 +849,17 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>2023
-(31/12/2023)</t>
+          <t>31/12/2023</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>2024
-(31/12/2024)</t>
+          <t>31/12/2024</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>2025
-(20/07/2025)*</t>
+          <t>20/07/2025*</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1014,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>RÉSULTAT EN COURS (exercice non clôturé)</t>
+          <t>RÉSULTAT EN COURS (exercice 2025 non clôturé)</t>
         </is>
       </c>
       <c r="B38" s="4" t="n"/>
@@ -1076,7 +1072,7 @@
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>* 2025 : exercice en cours, données au 20/07/2025 (non clôturé)</t>
+          <t>* 2025 : exercice en cours au 20/07/2025 (non clôturé)</t>
         </is>
       </c>
     </row>
@@ -1095,10 +1091,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -1107,7 +1103,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>COMPTE DE RÉSULTAT COMPARATIF PAR NATURE</t>
+          <t>COMPTE DE RÉSULTAT COMPARATIF PAR NATURE DE COMPTE</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1117,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>CHARGES PAR NATURE</t>
+          <t>CHARGES (Classe 6)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1188,11 +1184,11 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Sous-total Achats / Fluides</t>
+          <t>Sous-total 60 - Achats / Fluides</t>
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>5241.61</v>
+        <v>5241.610000000001</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1445.59</v>
@@ -1278,7 +1274,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6140 0023 - Contrat sécurité incendie</t>
+          <t xml:space="preserve">   6140 0023 - Contrat de sécurité incendie</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
@@ -1336,13 +1332,13 @@
         <v>138</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>140.48</v>
+        <v>-138</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>Sous-total Services extérieurs</t>
+          <t>Sous-total 61 - Services extérieurs</t>
         </is>
       </c>
       <c r="B19" s="13" t="n">
@@ -1352,13 +1348,13 @@
         <v>4186.25</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>1169.2</v>
+        <v>890.72</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>62 - AUTRES SERVICES EXTÉRIEURS</t>
+          <t>62 - AUTRES SERVICES EXTÉRIEURS (honoraires, frais juridiques)</t>
         </is>
       </c>
       <c r="B21" s="4" t="n"/>
@@ -1416,14 +1412,14 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6222 0001 - Vacations complémentaires</t>
+          <t xml:space="preserve">   6221 0201 - Honoraires travaux (AG Réso 22 haie)</t>
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="D25" s="6" t="n">
         <v>0</v>
@@ -1432,14 +1428,14 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6222 0002 - Réunions CS &amp; AG complémentaires</t>
+          <t xml:space="preserve">   6222 0001 - Vacations complémentaires</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>240</v>
+        <v>0</v>
       </c>
       <c r="C26" s="6" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="D26" s="6" t="n">
         <v>0</v>
@@ -1448,11 +1444,11 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6222 0005 - Pilotage et suivi contentieux</t>
+          <t xml:space="preserve">   6222 0002 - Réunions CS &amp; AG complémentaires</t>
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>1668</v>
+        <v>240</v>
       </c>
       <c r="C27" s="6" t="n">
         <v>0</v>
@@ -1464,11 +1460,11 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6230 0002 - Honoraires huissiers</t>
+          <t xml:space="preserve">   6222 0005 - Pilotage et suivi contentieux</t>
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>495.4</v>
+        <v>1668</v>
       </c>
       <c r="C28" s="6" t="n">
         <v>0</v>
@@ -1480,235 +1476,251 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">   6230 0002 - Honoraires huissiers</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>495.4</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">   6230 0003 - Honoraires avocats</t>
         </is>
       </c>
-      <c r="B29" s="6" t="n">
+      <c r="B30" s="6" t="n">
         <v>4500.08</v>
       </c>
-      <c r="C29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
-        <is>
-          <t>Sous-total Autres services extérieurs</t>
-        </is>
-      </c>
-      <c r="B30" s="13" t="n">
-        <v>8785.59</v>
-      </c>
-      <c r="C30" s="13" t="n">
-        <v>1969.4</v>
-      </c>
-      <c r="D30" s="13" t="n">
+      <c r="C30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>Sous-total 62 - Autres services extérieurs</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="n">
+        <v>8905.59</v>
+      </c>
+      <c r="C31" s="13" t="n">
+        <v>2089.4</v>
+      </c>
+      <c r="D31" s="13" t="n">
         <v>926.38</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>66 - CHARGES FINANCIÈRES</t>
         </is>
       </c>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   6620 0001 - Frais bancaires</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="n">
-        <v>286.54</v>
-      </c>
-      <c r="C33" s="6" t="n">
-        <v>96</v>
-      </c>
-      <c r="D33" s="6" t="n">
-        <v>72</v>
-      </c>
+      <c r="B33" s="4" t="n"/>
+      <c r="C33" s="4" t="n"/>
+      <c r="D33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">   6620 0001 - Frais bancaires</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>286.54</v>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>96</v>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">   6620 0002 - Reliquat de répartition (rompus)</t>
         </is>
       </c>
-      <c r="B34" s="6" t="n">
+      <c r="B35" s="6" t="n">
         <v>0.25</v>
       </c>
-      <c r="C34" s="6" t="n">
+      <c r="C35" s="6" t="n">
         <v>0.06</v>
       </c>
-      <c r="D34" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="12" t="inlineStr">
-        <is>
-          <t>Sous-total Charges financières</t>
-        </is>
-      </c>
-      <c r="B35" s="13" t="n">
+      <c r="D35" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>Sous-total 66 - Charges financières</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="n">
         <v>286.79</v>
       </c>
-      <c r="C35" s="13" t="n">
+      <c r="C36" s="13" t="n">
         <v>96.06</v>
       </c>
-      <c r="D35" s="13" t="n">
+      <c r="D36" s="13" t="n">
         <v>72</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>67 - CHARGES EXCEPTIONNELLES</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
-    </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>67 - CHARGES EXCEPTIONNELLES / TRAVAUX AG</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n"/>
+      <c r="C38" s="4" t="n"/>
+      <c r="D38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">   6780 0003 - Charges except. sur exercices antérieurs</t>
         </is>
       </c>
-      <c r="B38" s="6" t="n">
+      <c r="B39" s="6" t="n">
         <v>25.49</v>
       </c>
-      <c r="C38" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="12" t="inlineStr">
-        <is>
-          <t>Sous-total Charges exceptionnelles</t>
-        </is>
-      </c>
-      <c r="B39" s="13" t="n">
+      <c r="C39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   6710 0201 - Travaux décidés par l'AG (VMC/conduits)</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>792</v>
+      </c>
+      <c r="D40" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>Sous-total 67 - Charges exceptionnelles / Travaux</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="n">
         <v>25.49</v>
       </c>
-      <c r="C39" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="14" t="inlineStr">
-        <is>
-          <t>TOTAL CHARGES COURANTES</t>
-        </is>
-      </c>
-      <c r="B41" s="15" t="n">
-        <v>19066.03</v>
-      </c>
-      <c r="C41" s="15" t="n">
-        <v>7697.3</v>
-      </c>
-      <c r="D41" s="15" t="n">
-        <v>2437.55</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>CHARGES TRAVAUX (hors budget courant)</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="4" t="n"/>
-      <c r="D44" s="4" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   6221 0201 - Honoraires travaux (AG Réso 22 haie)</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="n">
-        <v>120</v>
-      </c>
-      <c r="C45" s="6" t="n">
-        <v>120</v>
-      </c>
-      <c r="D45" s="6" t="n">
-        <v>0</v>
+      <c r="C41" s="13" t="n">
+        <v>792</v>
+      </c>
+      <c r="D41" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>TOTAL CHARGES (Classe 6)</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="n">
+        <v>19186.03</v>
+      </c>
+      <c r="C43" s="15" t="n">
+        <v>8609.299999999999</v>
+      </c>
+      <c r="D43" s="15" t="n">
+        <v>2159.07</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   6710 0201 - Travaux décidés par l'AG (VMC/conduits)</t>
-        </is>
-      </c>
-      <c r="B46" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C46" s="6" t="n">
-        <v>792</v>
-      </c>
-      <c r="D46" s="6" t="n">
-        <v>0</v>
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>PRODUITS (Classe 7)</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>2025*</t>
+        </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="16" t="inlineStr">
-        <is>
-          <t>TOTAL CHARGES TRAVAUX</t>
-        </is>
-      </c>
-      <c r="B47" s="17" t="n">
-        <v>120</v>
-      </c>
-      <c r="C47" s="17" t="n">
-        <v>912</v>
-      </c>
-      <c r="D47" s="17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>PRODUITS PAR NATURE</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>2025*</t>
-        </is>
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>70 - PROVISIONS POUR CHARGES COURANTES</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="n"/>
+      <c r="C47" s="4" t="n"/>
+      <c r="D47" s="4" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   7010 - Provisions sur opérations courantes</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="n">
+        <v>18000</v>
+      </c>
+      <c r="C48" s="6" t="n">
+        <v>16000</v>
+      </c>
+      <c r="D48" s="6" t="n">
+        <v>10274.94</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>Sous-total 70 - Provisions</t>
+        </is>
+      </c>
+      <c r="B49" s="13" t="n">
+        <v>18000</v>
+      </c>
+      <c r="C49" s="13" t="n">
+        <v>16000</v>
+      </c>
+      <c r="D49" s="13" t="n">
+        <v>10274.94</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>70 - PROVISIONS POUR CHARGES</t>
+          <t>71 - PRODUITS EXCEPTIONNELS</t>
         </is>
       </c>
       <c r="B51" s="4" t="n"/>
@@ -1718,172 +1730,130 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   7010 - Provisions sur opérations courantes</t>
+          <t xml:space="preserve">   7180 - Produits exceptionnels (FNP antérieures)</t>
         </is>
       </c>
       <c r="B52" s="6" t="n">
-        <v>18000</v>
+        <v>400</v>
       </c>
       <c r="C52" s="6" t="n">
-        <v>16000</v>
+        <v>0</v>
       </c>
       <c r="D52" s="6" t="n">
-        <v>10274.94</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t>Sous-total Provisions</t>
+          <t>Sous-total 71 - Produits exceptionnels</t>
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>18000</v>
+        <v>400</v>
       </c>
       <c r="C53" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL PRODUITS (Classe 7)</t>
+        </is>
+      </c>
+      <c r="B55" s="17" t="n">
+        <v>18400</v>
+      </c>
+      <c r="C55" s="17" t="n">
         <v>16000</v>
       </c>
-      <c r="D53" s="13" t="n">
+      <c r="D55" s="17" t="n">
         <v>10274.94</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>71 - PRODUITS EXCEPTIONNELS</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="4" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   7180 - Produits exceptionnels</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="C56" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D56" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="12" t="inlineStr">
-        <is>
-          <t>Sous-total Produits exceptionnels</t>
-        </is>
-      </c>
-      <c r="B57" s="13" t="n">
-        <v>400</v>
-      </c>
-      <c r="C57" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D57" s="13" t="n">
-        <v>0</v>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>RÉSULTAT DE L'EXERCICE</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>2025*</t>
+        </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="18" t="inlineStr">
         <is>
-          <t>TOTAL PRODUITS</t>
+          <t>Résultat = Produits (Cl. 7) - Charges (Cl. 6)</t>
         </is>
       </c>
       <c r="B59" s="19" t="n">
-        <v>18400</v>
+        <v>-786.0299999999988</v>
       </c>
       <c r="C59" s="19" t="n">
-        <v>16000</v>
+        <v>7390.700000000001</v>
       </c>
       <c r="D59" s="19" t="n">
-        <v>10274.94</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>RÉSULTAT DE L'EXERCICE</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>2025*</t>
-        </is>
+        <v>8115.870000000001</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="20" t="inlineStr">
+        <is>
+          <t>Excédent (+) ou Déficit (-)</t>
+        </is>
+      </c>
+      <c r="B61" s="21" t="n">
+        <v>-786.0299999999988</v>
+      </c>
+      <c r="C61" s="21" t="n">
+        <v>7390.700000000001</v>
+      </c>
+      <c r="D61" s="21" t="n">
+        <v>8115.870000000001</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="9" t="inlineStr">
-        <is>
-          <t>Résultat courant (Produits - Charges courantes)</t>
-        </is>
-      </c>
-      <c r="B63" s="10" t="n">
-        <v>-666.0300000000025</v>
-      </c>
-      <c r="C63" s="10" t="n">
-        <v>8302.700000000001</v>
-      </c>
-      <c r="D63" s="10" t="n">
-        <v>7837.39</v>
+      <c r="A63" s="22" t="inlineStr">
+        <is>
+          <t>Résultat positif = excédent (provisions &gt; charges réelles).</t>
+        </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="7" t="inlineStr">
-        <is>
-          <t>Résultat = Excédent (+) / Déficit (-)</t>
-        </is>
-      </c>
-      <c r="B64" s="8" t="n">
-        <v>-666.0300000000025</v>
-      </c>
-      <c r="C64" s="8" t="n">
-        <v>8302.700000000001</v>
-      </c>
-      <c r="D64" s="8" t="n">
-        <v>7837.39</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="11" t="inlineStr">
-        <is>
-          <t>Un résultat positif = excédent (provisions &gt; charges).</t>
+      <c r="A64" s="22" t="inlineStr">
+        <is>
+          <t>Résultat négatif = déficit (charges réelles &gt; provisions appelées).</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="11" t="inlineStr">
-        <is>
-          <t>Un résultat négatif = déficit (charges &gt; provisions).</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="20" t="inlineStr">
-        <is>
-          <t>* 2025 : exercice en cours au 20/07/2025, données partielles (6 mois et demi)</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="11" t="inlineStr">
-        <is>
-          <t>Note : les charges travaux (6221/6710) sont hors budget courant et font l'objet d'appels spécifiques.</t>
+      <c r="A66" s="23" t="inlineStr">
+        <is>
+          <t>* 2025 : exercice en cours au 20/07/2025, données partielles (~6,5 mois).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="22" t="inlineStr">
+        <is>
+          <t>Note : les frais privatifs (mutations, mises en demeure) transitent en débit/crédit et n'affectent pas le résultat.</t>
         </is>
       </c>
     </row>
@@ -1894,436 +1864,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>DÉTAIL DU BILAN PAR COMPTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="21" t="inlineStr">
-        <is>
-          <t>Compte</t>
-        </is>
-      </c>
-      <c r="B3" s="21" t="inlineStr">
-        <is>
-          <t>Libellé</t>
-        </is>
-      </c>
-      <c r="C3" s="21" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="D3" s="21" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="E3" s="21" t="inlineStr">
-        <is>
-          <t>2025*</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="22" t="inlineStr"/>
-      <c r="B4" s="22" t="inlineStr">
-        <is>
-          <t>ACTIF</t>
-        </is>
-      </c>
-      <c r="C4" s="23" t="n"/>
-      <c r="D4" s="23" t="n"/>
-      <c r="E4" s="23" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="24" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="B5" s="24" t="inlineStr">
-        <is>
-          <t>Solde en attente sur travaux</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>120</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="24" t="inlineStr">
-        <is>
-          <t>4010</t>
-        </is>
-      </c>
-      <c r="B6" s="24" t="inlineStr">
-        <is>
-          <t>Fournisseurs débiteurs</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>278.48</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="24" t="inlineStr">
-        <is>
-          <t>450</t>
-        </is>
-      </c>
-      <c r="B7" s="24" t="inlineStr">
-        <is>
-          <t>Copropriétaires débiteurs</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>3776.31</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="24" t="inlineStr">
-        <is>
-          <t>4711</t>
-        </is>
-      </c>
-      <c r="B8" s="24" t="inlineStr">
-        <is>
-          <t>Régularisation charges - Débiteur</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>18665.97</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>26363.21</v>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>26363.21</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="24" t="inlineStr">
-        <is>
-          <t>4712</t>
-        </is>
-      </c>
-      <c r="B9" s="24" t="inlineStr">
-        <is>
-          <t>Régularisation travaux - Débiteur</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>911.97</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>911.97</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="24" t="inlineStr">
-        <is>
-          <t>4730</t>
-        </is>
-      </c>
-      <c r="B10" s="24" t="inlineStr">
-        <is>
-          <t>Rompus débiteurs</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="24" t="inlineStr">
-        <is>
-          <t>5120 0001</t>
-        </is>
-      </c>
-      <c r="B11" s="24" t="inlineStr">
-        <is>
-          <t>Compte courant Montepaschi</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>2968.03</v>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>9525.9</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>13074.46</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="24" t="inlineStr">
-        <is>
-          <t>5120 0004</t>
-        </is>
-      </c>
-      <c r="B12" s="24" t="inlineStr">
-        <is>
-          <t>Livret A Monte Paschi</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>910.22</v>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>1742.55</v>
-      </c>
-      <c r="E12" s="6" t="n">
-        <v>1967.53</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="22" t="inlineStr"/>
-      <c r="B13" s="22" t="inlineStr">
-        <is>
-          <t>TOTAL ACTIF</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>22664.28</v>
-      </c>
-      <c r="D13" s="8" t="n">
-        <v>38543.72</v>
-      </c>
-      <c r="E13" s="8" t="n">
-        <v>46372.05</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="24" t="inlineStr"/>
-      <c r="B14" s="24" t="inlineStr"/>
-      <c r="C14" s="25" t="n"/>
-      <c r="D14" s="25" t="n"/>
-      <c r="E14" s="25" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="22" t="inlineStr"/>
-      <c r="B15" s="22" t="inlineStr">
-        <is>
-          <t>PASSIF</t>
-        </is>
-      </c>
-      <c r="C15" s="23" t="n"/>
-      <c r="D15" s="23" t="n"/>
-      <c r="E15" s="23" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="24" t="inlineStr">
-        <is>
-          <t>1031</t>
-        </is>
-      </c>
-      <c r="B16" s="24" t="inlineStr">
-        <is>
-          <t>Avances de trésorerie</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>2000</v>
-      </c>
-      <c r="D16" s="6" t="n">
-        <v>2000</v>
-      </c>
-      <c r="E16" s="6" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="24" t="inlineStr">
-        <is>
-          <t>1050</t>
-        </is>
-      </c>
-      <c r="B17" s="24" t="inlineStr">
-        <is>
-          <t>Fonds de travaux</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="n">
-        <v>910.22</v>
-      </c>
-      <c r="D17" s="6" t="n">
-        <v>1742.55</v>
-      </c>
-      <c r="E17" s="6" t="n">
-        <v>2256.18</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="24" t="inlineStr">
-        <is>
-          <t>4010</t>
-        </is>
-      </c>
-      <c r="B18" s="24" t="inlineStr">
-        <is>
-          <t>Fournisseurs créditeurs</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>1330.06</v>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>659.45</v>
-      </c>
-      <c r="E18" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="24" t="inlineStr">
-        <is>
-          <t>4080</t>
-        </is>
-      </c>
-      <c r="B19" s="24" t="inlineStr">
-        <is>
-          <t>Factures non parvenues</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>141.72</v>
-      </c>
-      <c r="E19" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="24" t="inlineStr">
-        <is>
-          <t>4630</t>
-        </is>
-      </c>
-      <c r="B20" s="24" t="inlineStr">
-        <is>
-          <t>Tiers créditeurs (anciens copro)</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>424</v>
-      </c>
-      <c r="D20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="24" t="inlineStr">
-        <is>
-          <t>4721</t>
-        </is>
-      </c>
-      <c r="B21" s="24" t="inlineStr">
-        <is>
-          <t>Régularisation charges - Créditeur</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>18000</v>
-      </c>
-      <c r="D21" s="6" t="n">
-        <v>34000</v>
-      </c>
-      <c r="E21" s="6" t="n">
-        <v>34000</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="24" t="inlineStr"/>
-      <c r="B22" s="24" t="inlineStr">
-        <is>
-          <t>Résultat en cours (classe 6 &amp; 7)</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="6" t="n">
-        <v>8115.87</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="22" t="inlineStr"/>
-      <c r="B23" s="22" t="inlineStr">
-        <is>
-          <t>TOTAL PASSIF</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="n">
-        <v>22664.28</v>
-      </c>
-      <c r="D23" s="8" t="n">
-        <v>38543.72</v>
-      </c>
-      <c r="E23" s="8" t="n">
-        <v>46372.05</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Bilan classique Actif/Passif côte à côte avec couleurs et résultat net
- Bilan présenté en format classique : Actif (bleu) à gauche, Passif (orange) à droite
- Résultat net inscrit au passif pour équilibrer le bilan
- Pour 2023/2024 clôturés, résultat déjà intégré dans les comptes 4711/4721
- Pour 2025 en cours, résultat (Produits - Charges) ajouté au passif
- Bilan équilibré sur les 3 exercices : vérification automatique
- Design coloré : sections, sous-totaux, totaux généraux
- Contrôle d'équilibre affiché en bas du bilan

Co-authored-by: alainannickbaptiste-dot <alainannickbaptiste-dot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/bilan_comptable_comparatif.xlsx
+++ b/bilan_comptable_comparatif.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,8 +80,28 @@
       <color rgb="00FF0000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00006100"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -126,8 +146,44 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B4C6E7"/>
-        <bgColor rgb="00B4C6E7"/>
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00404040"/>
+        <bgColor rgb="00404040"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00833C0B"/>
+        <bgColor rgb="00833C0B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009DC3E6"/>
+        <bgColor rgb="009DC3E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -149,7 +205,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -196,11 +252,60 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1328,726 +1433,635 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="55" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>BILAN COMPARATIF - Mouvements de l'exercice</t>
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>BILAN COMPARATIF</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>SDC 17 Rue Léon Cladel, Sèvres - Copropriété PERDUE</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Compte / Libellé</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>2023
-Débit - Crédit</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>2024
-Débit - Crédit</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>2025*
-Débit - Crédit</t>
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>ACTIF</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>2025*</t>
+        </is>
+      </c>
+      <c r="E4" s="21" t="n"/>
+      <c r="F4" s="22" t="inlineStr">
+        <is>
+          <t>PASSIF</t>
+        </is>
+      </c>
+      <c r="G4" s="22" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="H4" s="22" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="I4" s="22" t="inlineStr">
+        <is>
+          <t>2025*</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Classe 1 - CAPITAUX ET PROVISIONS</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>Actif immobilisé</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="inlineStr"/>
+      <c r="C5" s="23" t="inlineStr"/>
+      <c r="D5" s="23" t="inlineStr"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="24" t="inlineStr">
+        <is>
+          <t>Avances et fonds de travaux</t>
+        </is>
+      </c>
+      <c r="G5" s="24" t="inlineStr"/>
+      <c r="H5" s="24" t="inlineStr"/>
+      <c r="I5" s="24" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   1031 0001 - Avances de trésorerie</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>0</v>
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Solde en attente travaux (1200)</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="n">
+        <v>120</v>
+      </c>
+      <c r="C6" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Avances de trésorerie (1031)</t>
+        </is>
+      </c>
+      <c r="G6" s="26" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H6" s="26" t="n">
+        <v>2000</v>
+      </c>
+      <c r="I6" s="26" t="n">
+        <v>2000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   1050 0001 - Fonds de travaux</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>-900.15</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>-832.33</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>-513.63</v>
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Total Actif immobilisé</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="n">
+        <v>120</v>
+      </c>
+      <c r="C7" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Fonds de travaux (1050)</t>
+        </is>
+      </c>
+      <c r="G7" s="26" t="n">
+        <v>910.22</v>
+      </c>
+      <c r="H7" s="26" t="n">
+        <v>1742.55</v>
+      </c>
+      <c r="I7" s="26" t="n">
+        <v>2256.18</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   1200 0002 - Solde en attente sur travaux et opérations</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>0</v>
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>Créances copropriétaires (450)</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr"/>
+      <c r="C8" s="23" t="inlineStr"/>
+      <c r="D8" s="23" t="inlineStr"/>
+      <c r="E8" s="21" t="n"/>
+      <c r="F8" s="29" t="inlineStr">
+        <is>
+          <t>Total Avances et fonds de travaux</t>
+        </is>
+      </c>
+      <c r="G8" s="30" t="n">
+        <v>2910.22</v>
+      </c>
+      <c r="H8" s="30" t="n">
+        <v>3742.55</v>
+      </c>
+      <c r="I8" s="30" t="n">
+        <v>4256.18</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Total Classe 1 - CAPITAUX ET PROVISIONS</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="n">
-        <v>-900.15</v>
-      </c>
-      <c r="C9" s="19" t="n">
-        <v>-832.33</v>
-      </c>
-      <c r="D9" s="19" t="n">
-        <v>-513.63</v>
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Copropriétaires - soldes débiteurs</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>3776.31</v>
+      </c>
+      <c r="E9" s="21" t="n"/>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>Dettes fournisseurs</t>
+        </is>
+      </c>
+      <c r="G9" s="24" t="inlineStr"/>
+      <c r="H9" s="24" t="inlineStr"/>
+      <c r="I9" s="24" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>Total Créances copropriétaires (450)</t>
+        </is>
+      </c>
+      <c r="B10" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="28" t="n">
+        <v>3776.31</v>
+      </c>
+      <c r="E10" s="21" t="n"/>
+      <c r="F10" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Fournisseurs créditeurs (4010)</t>
+        </is>
+      </c>
+      <c r="G10" s="26" t="n">
+        <v>1330.06</v>
+      </c>
+      <c r="H10" s="26" t="n">
+        <v>659.45</v>
+      </c>
+      <c r="I10" s="26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Classe 4 - TIERS</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>Créances fournisseurs &amp; tiers</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="inlineStr"/>
+      <c r="C11" s="23" t="inlineStr"/>
+      <c r="D11" s="23" t="inlineStr"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Factures non parvenues (4080)</t>
+        </is>
+      </c>
+      <c r="G11" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="26" t="n">
+        <v>141.72</v>
+      </c>
+      <c r="I11" s="26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0002 - 2S2P PROFESSIONNEL - Nettoyage courant des</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>11.49999999999955</v>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>261.6</v>
-      </c>
-      <c r="D12" s="7" t="n">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Fournisseurs débiteurs (4010)</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="26" t="n">
+        <v>278.48</v>
+      </c>
+      <c r="E12" s="21" t="n"/>
+      <c r="F12" s="29" t="inlineStr">
+        <is>
+          <t>Total Dettes fournisseurs</t>
+        </is>
+      </c>
+      <c r="G12" s="30" t="n">
+        <v>1330.06</v>
+      </c>
+      <c r="H12" s="30" t="n">
+        <v>801.1700000000001</v>
+      </c>
+      <c r="I12" s="30" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0003 - MANDA (Ex Hello Syndic) - HELLO SYNDIC</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="n">
-        <v>3961.23</v>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>-70.12999999999965</v>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>70.13000000000011</v>
-      </c>
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>Total Créances fournisseurs &amp; tiers</t>
+        </is>
+      </c>
+      <c r="B13" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="28" t="n">
+        <v>278.48</v>
+      </c>
+      <c r="E13" s="21" t="n"/>
+      <c r="F13" s="24" t="inlineStr">
+        <is>
+          <t>Dettes et tiers créditeurs</t>
+        </is>
+      </c>
+      <c r="G13" s="24" t="inlineStr"/>
+      <c r="H13" s="24" t="inlineStr"/>
+      <c r="I13" s="24" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0005 - P Plasse</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="7" t="n">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>Comptes de régularisation - Actif</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="inlineStr"/>
+      <c r="C14" s="23" t="inlineStr"/>
+      <c r="D14" s="23" t="inlineStr"/>
+      <c r="E14" s="21" t="n"/>
+      <c r="F14" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Anciens copropriétaires (4630)</t>
+        </is>
+      </c>
+      <c r="G14" s="26" t="n">
+        <v>424</v>
+      </c>
+      <c r="H14" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0006 - AUDREY BENOIS</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="7" t="n">
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Régularisation charges débiteur (4711)</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="n">
+        <v>18665.97</v>
+      </c>
+      <c r="C15" s="26" t="n">
+        <v>26363.21</v>
+      </c>
+      <c r="D15" s="26" t="n">
+        <v>26363.21</v>
+      </c>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="29" t="inlineStr">
+        <is>
+          <t>Total Dettes et tiers créditeurs</t>
+        </is>
+      </c>
+      <c r="G15" s="30" t="n">
+        <v>424</v>
+      </c>
+      <c r="H15" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="30" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0007 - VEOLIA - 1495884 - Contrat résilié à partir 01/01/</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="n">
-        <v>-493.9599999999999</v>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>841.4899999999998</v>
-      </c>
-      <c r="D16" s="7" t="n">
-        <v>226.97</v>
-      </c>
+      <c r="A16" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Régularisation travaux débiteur (4712)</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="26" t="n">
+        <v>911.97</v>
+      </c>
+      <c r="D16" s="26" t="n">
+        <v>911.97</v>
+      </c>
+      <c r="E16" s="21" t="n"/>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>Comptes de régularisation - Passif</t>
+        </is>
+      </c>
+      <c r="G16" s="24" t="inlineStr"/>
+      <c r="H16" s="24" t="inlineStr"/>
+      <c r="I16" s="24" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0008 - EDF Entreprises - [Prlv] contrat 8300132433</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="n">
-        <v>2869.610000000001</v>
-      </c>
-      <c r="C17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>0</v>
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Rompus débiteurs (4730)</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C17" s="26" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="D17" s="26" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E17" s="21" t="n"/>
+      <c r="F17" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Régularisation charges créditeur (4721)</t>
+        </is>
+      </c>
+      <c r="G17" s="26" t="n">
+        <v>18000</v>
+      </c>
+      <c r="H17" s="26" t="n">
+        <v>34000</v>
+      </c>
+      <c r="I17" s="26" t="n">
+        <v>34000</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0009 - PRO ARCHIVES</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="7" t="n">
-        <v>0</v>
+      <c r="A18" s="27" t="inlineStr">
+        <is>
+          <t>Total Comptes de régularisation - Actif</t>
+        </is>
+      </c>
+      <c r="B18" s="28" t="n">
+        <v>18666.03</v>
+      </c>
+      <c r="C18" s="28" t="n">
+        <v>27275.27</v>
+      </c>
+      <c r="D18" s="28" t="n">
+        <v>27275.27</v>
+      </c>
+      <c r="E18" s="21" t="n"/>
+      <c r="F18" s="29" t="inlineStr">
+        <is>
+          <t>Total Comptes de régularisation - Passif</t>
+        </is>
+      </c>
+      <c r="G18" s="30" t="n">
+        <v>18000</v>
+      </c>
+      <c r="H18" s="30" t="n">
+        <v>34000</v>
+      </c>
+      <c r="I18" s="30" t="n">
+        <v>34000</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0021 - DIDIER &amp; XAVIER - AVALLE ASSOCIES</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>Trésorerie</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="inlineStr"/>
+      <c r="C19" s="23" t="inlineStr"/>
+      <c r="D19" s="23" t="inlineStr"/>
+      <c r="E19" s="21" t="n"/>
+      <c r="F19" s="25" t="inlineStr"/>
+      <c r="G19" s="25" t="inlineStr"/>
+      <c r="H19" s="25" t="inlineStr"/>
+      <c r="I19" s="25" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0022 - AIAC</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="A20" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Compte courant Montepaschi</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="n">
+        <v>2968.03</v>
+      </c>
+      <c r="C20" s="26" t="n">
+        <v>9525.9</v>
+      </c>
+      <c r="D20" s="26" t="n">
+        <v>13074.46</v>
+      </c>
+      <c r="E20" s="21" t="n"/>
+      <c r="F20" s="25" t="inlineStr"/>
+      <c r="G20" s="25" t="inlineStr"/>
+      <c r="H20" s="25" t="inlineStr"/>
+      <c r="I20" s="25" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0023 - ATLAS JUSTICE</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="A21" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Livret A Monte Paschi</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="n">
+        <v>910.22</v>
+      </c>
+      <c r="C21" s="26" t="n">
+        <v>1742.55</v>
+      </c>
+      <c r="D21" s="26" t="n">
+        <v>1967.53</v>
+      </c>
+      <c r="E21" s="21" t="n"/>
+      <c r="F21" s="25" t="inlineStr"/>
+      <c r="G21" s="25" t="inlineStr"/>
+      <c r="H21" s="25" t="inlineStr"/>
+      <c r="I21" s="25" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0024 - EDF contrat 5342619275</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="n">
-        <v>99.12</v>
-      </c>
-      <c r="C22" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0026 - REALBA ETANCHEITE</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C23" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="A22" s="27" t="inlineStr">
+        <is>
+          <t>Total Trésorerie</t>
+        </is>
+      </c>
+      <c r="B22" s="28" t="n">
+        <v>3878.25</v>
+      </c>
+      <c r="C22" s="28" t="n">
+        <v>11268.45</v>
+      </c>
+      <c r="D22" s="28" t="n">
+        <v>15041.99</v>
+      </c>
+      <c r="E22" s="21" t="n"/>
+      <c r="F22" s="25" t="inlineStr"/>
+      <c r="G22" s="25" t="inlineStr"/>
+      <c r="H22" s="25" t="inlineStr"/>
+      <c r="I22" s="25" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0028 - BOUVIER</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C24" s="7" t="n">
-        <v>-362.35</v>
-      </c>
-      <c r="D24" s="7" t="n">
-        <v>362.35</v>
+      <c r="A24" s="25" t="inlineStr"/>
+      <c r="B24" s="25" t="inlineStr"/>
+      <c r="C24" s="25" t="inlineStr"/>
+      <c r="D24" s="25" t="inlineStr"/>
+      <c r="E24" s="21" t="n"/>
+      <c r="F24" s="31" t="inlineStr">
+        <is>
+          <t>Résultat net de l'exercice</t>
+        </is>
+      </c>
+      <c r="G24" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="33" t="n">
+        <v>8115.870000000001</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0029 - AUTOTROPHE PAYSAGE</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="E25" s="21" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0030 - AVIPUR</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0031 - PHERELEC Électricité</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="7" t="n">
-        <v>0</v>
+      <c r="A26" s="34" t="inlineStr">
+        <is>
+          <t>TOTAL ACTIF</t>
+        </is>
+      </c>
+      <c r="B26" s="35" t="n">
+        <v>22664.28</v>
+      </c>
+      <c r="C26" s="35" t="n">
+        <v>38543.72</v>
+      </c>
+      <c r="D26" s="35" t="n">
+        <v>46372.05</v>
+      </c>
+      <c r="E26" s="21" t="n"/>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>TOTAL PASSIF</t>
+        </is>
+      </c>
+      <c r="G26" s="35" t="n">
+        <v>22664.28</v>
+      </c>
+      <c r="H26" s="35" t="n">
+        <v>38543.72</v>
+      </c>
+      <c r="I26" s="35" t="n">
+        <v>46372.05</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0032 - SCI ZADOM</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="7" t="n">
-        <v>0</v>
+      <c r="A28" s="36" t="inlineStr">
+        <is>
+          <t>Contrôle 2023: ✓ Équilibré</t>
+        </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0033 - SOGECOP</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="7" t="n">
-        <v>0</v>
+      <c r="A29" s="36" t="inlineStr">
+        <is>
+          <t>Contrôle 2024: ✓ Équilibré</t>
+        </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0035 - FILHET-ALLARD - Courtier assurance</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="7" t="n">
-        <v>278.48</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4010 0036 - L'EAU D'ILE-DE-FRANCE</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C31" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="7" t="n">
-        <v>0</v>
+      <c r="A30" s="36" t="inlineStr">
+        <is>
+          <t>Contrôle 2025: ✓ Équilibré</t>
+        </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4080 0001 - Factures non parvenues</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="n">
-        <v>1609.92</v>
-      </c>
-      <c r="C32" s="7" t="n">
-        <v>-141.7200000000084</v>
-      </c>
-      <c r="D32" s="7" t="n">
-        <v>3918.029999999997</v>
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>* 2025 : exercice en cours au 20/07/2025 (non clôturé).</t>
+        </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4310 0001 - URSSAF - Sécurité sociale</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="n">
-        <v>-573</v>
-      </c>
-      <c r="C33" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4320 1002 - HUMANIS PREVOYANCE - Organisme</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="n">
-        <v>-8.359999999999999</v>
-      </c>
-      <c r="C34" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4320 3003 - HUMANIS RETRAITE - Organisme retraite</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="n">
-        <v>-4853.229999999992</v>
-      </c>
-      <c r="C35" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4630 0004 - Azzopardi - Ancien copropriétaire</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C36" s="7" t="n">
-        <v>424</v>
-      </c>
-      <c r="D36" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4711 0001 - Régularisation des charges - Débiteur</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="n">
-        <v>-57371.18</v>
-      </c>
-      <c r="C37" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4712 0001 - Régularisation des travaux - Débiteur - AG 2018</t>
-        </is>
-      </c>
-      <c r="B38" s="7" t="n">
-        <v>-3553.85</v>
-      </c>
-      <c r="C38" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4712 0002 - Régularisation des travaux - Débiteur - AG 19/</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C39" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4721 0001 - Régularisation des charges - Créditeur</t>
-        </is>
-      </c>
-      <c r="B40" s="7" t="n">
-        <v>54000</v>
-      </c>
-      <c r="C40" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4722 0001 - Régularisation des travaux - Créditeur - AG 2018</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="n">
-        <v>3553.88</v>
-      </c>
-      <c r="C41" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D41" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   4730 0000 - Rompus</t>
-        </is>
-      </c>
-      <c r="B42" s="7" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="C42" s="7" t="n">
-        <v>-0.06</v>
-      </c>
-      <c r="D42" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="18" t="inlineStr">
-        <is>
-          <t>Total Classe 4 - TIERS</t>
-        </is>
-      </c>
-      <c r="B43" s="19" t="n">
-        <v>-748.5699999999897</v>
-      </c>
-      <c r="C43" s="19" t="n">
-        <v>952.8299999999916</v>
-      </c>
-      <c r="D43" s="19" t="n">
-        <v>4855.959999999997</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>Classe 5 - TRÉSORERIE</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="n"/>
-      <c r="C45" s="5" t="n"/>
-      <c r="D45" s="5" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   5120 0001 - Compte courant Montepaschi - SDC DU 17 RUE</t>
-        </is>
-      </c>
-      <c r="B46" s="7" t="n">
-        <v>-47.53000000000611</v>
-      </c>
-      <c r="C46" s="7" t="n">
-        <v>6557.870000000001</v>
-      </c>
-      <c r="D46" s="7" t="n">
-        <v>3548.559999999999</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   5120 0004 - Livret A Monte Paschi - LIVRET A 17 RUE LEON</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="n">
-        <v>910.22</v>
-      </c>
-      <c r="C47" s="7" t="n">
-        <v>832.3299999999999</v>
-      </c>
-      <c r="D47" s="7" t="n">
-        <v>224.98</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="18" t="inlineStr">
-        <is>
-          <t>Total Classe 5 - TRÉSORERIE</t>
-        </is>
-      </c>
-      <c r="B48" s="19" t="n">
-        <v>862.6899999999939</v>
-      </c>
-      <c r="C48" s="19" t="n">
-        <v>7390.200000000001</v>
-      </c>
-      <c r="D48" s="19" t="n">
-        <v>3773.54</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="16" t="inlineStr">
-        <is>
-          <t>Solde positif = débiteur (actif) | Solde négatif = créditeur (passif)</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="17" t="inlineStr">
-        <is>
-          <t>* 2025 : exercice en cours au 20/07/2025.</t>
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>Le résultat net est inscrit au passif pour équilibrer le bilan (excédent = passif / déficit = diminue le passif).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2140,12 +2154,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="37" t="inlineStr">
         <is>
           <t>1031 0001</t>
         </is>
       </c>
-      <c r="B4" s="21" t="inlineStr">
+      <c r="B4" s="38" t="inlineStr">
         <is>
           <t>Avances de trésorerie</t>
         </is>
@@ -2179,12 +2193,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="37" t="inlineStr">
         <is>
           <t>1050 0001</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="38" t="inlineStr">
         <is>
           <t>Fonds de travaux</t>
         </is>
@@ -2218,12 +2232,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t>1200 0002</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="38" t="inlineStr">
         <is>
           <t>Solde en attente sur travaux et opérations</t>
         </is>
@@ -2257,12 +2271,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="37" t="inlineStr">
         <is>
           <t>4010 0002</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="38" t="inlineStr">
         <is>
           <t>2S2P PROFESSIONNEL - Nettoyage courant des</t>
         </is>
@@ -2296,12 +2310,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="37" t="inlineStr">
         <is>
           <t>4010 0003</t>
         </is>
       </c>
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="38" t="inlineStr">
         <is>
           <t>MANDA (Ex Hello Syndic) - HELLO SYNDIC</t>
         </is>
@@ -2335,12 +2349,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t>4010 0005</t>
         </is>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B9" s="38" t="inlineStr">
         <is>
           <t>P Plasse</t>
         </is>
@@ -2374,12 +2388,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t>4010 0006</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>AUDREY BENOIS</t>
         </is>
@@ -2413,12 +2427,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="37" t="inlineStr">
         <is>
           <t>4010 0007</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="38" t="inlineStr">
         <is>
           <t>VEOLIA - 1495884 - Contrat résilié à partir 01/01/</t>
         </is>
@@ -2452,12 +2466,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="37" t="inlineStr">
         <is>
           <t>4010 0008</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="38" t="inlineStr">
         <is>
           <t>EDF Entreprises - [Prlv] contrat 8300132433</t>
         </is>
@@ -2491,12 +2505,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="37" t="inlineStr">
         <is>
           <t>4010 0009</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B13" s="38" t="inlineStr">
         <is>
           <t>PRO ARCHIVES</t>
         </is>
@@ -2530,12 +2544,12 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="A14" s="37" t="inlineStr">
         <is>
           <t>4010 0021</t>
         </is>
       </c>
-      <c r="B14" s="21" t="inlineStr">
+      <c r="B14" s="38" t="inlineStr">
         <is>
           <t>DIDIER &amp; XAVIER - AVALLE ASSOCIES</t>
         </is>
@@ -2569,12 +2583,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="37" t="inlineStr">
         <is>
           <t>4010 0022</t>
         </is>
       </c>
-      <c r="B15" s="21" t="inlineStr">
+      <c r="B15" s="38" t="inlineStr">
         <is>
           <t>AIAC</t>
         </is>
@@ -2608,12 +2622,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="37" t="inlineStr">
         <is>
           <t>4010 0023</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="38" t="inlineStr">
         <is>
           <t>ATLAS JUSTICE</t>
         </is>
@@ -2647,12 +2661,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="37" t="inlineStr">
         <is>
           <t>4010 0024</t>
         </is>
       </c>
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B17" s="38" t="inlineStr">
         <is>
           <t>EDF contrat 5342619275</t>
         </is>
@@ -2686,12 +2700,12 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" s="37" t="inlineStr">
         <is>
           <t>4010 0026</t>
         </is>
       </c>
-      <c r="B18" s="21" t="inlineStr">
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>REALBA ETANCHEITE</t>
         </is>
@@ -2725,12 +2739,12 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="20" t="inlineStr">
+      <c r="A19" s="37" t="inlineStr">
         <is>
           <t>4010 0028</t>
         </is>
       </c>
-      <c r="B19" s="21" t="inlineStr">
+      <c r="B19" s="38" t="inlineStr">
         <is>
           <t>BOUVIER</t>
         </is>
@@ -2764,12 +2778,12 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="inlineStr">
+      <c r="A20" s="37" t="inlineStr">
         <is>
           <t>4010 0029</t>
         </is>
       </c>
-      <c r="B20" s="21" t="inlineStr">
+      <c r="B20" s="38" t="inlineStr">
         <is>
           <t>AUTOTROPHE PAYSAGE</t>
         </is>
@@ -2803,12 +2817,12 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A21" s="37" t="inlineStr">
         <is>
           <t>4010 0030</t>
         </is>
       </c>
-      <c r="B21" s="21" t="inlineStr">
+      <c r="B21" s="38" t="inlineStr">
         <is>
           <t>AVIPUR</t>
         </is>
@@ -2842,12 +2856,12 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="20" t="inlineStr">
+      <c r="A22" s="37" t="inlineStr">
         <is>
           <t>4010 0031</t>
         </is>
       </c>
-      <c r="B22" s="21" t="inlineStr">
+      <c r="B22" s="38" t="inlineStr">
         <is>
           <t>PHERELEC Électricité</t>
         </is>
@@ -2881,12 +2895,12 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="inlineStr">
+      <c r="A23" s="37" t="inlineStr">
         <is>
           <t>4010 0032</t>
         </is>
       </c>
-      <c r="B23" s="21" t="inlineStr">
+      <c r="B23" s="38" t="inlineStr">
         <is>
           <t>SCI ZADOM</t>
         </is>
@@ -2920,12 +2934,12 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="20" t="inlineStr">
+      <c r="A24" s="37" t="inlineStr">
         <is>
           <t>4010 0033</t>
         </is>
       </c>
-      <c r="B24" s="21" t="inlineStr">
+      <c r="B24" s="38" t="inlineStr">
         <is>
           <t>SOGECOP</t>
         </is>
@@ -2959,12 +2973,12 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="20" t="inlineStr">
+      <c r="A25" s="37" t="inlineStr">
         <is>
           <t>4010 0035</t>
         </is>
       </c>
-      <c r="B25" s="21" t="inlineStr">
+      <c r="B25" s="38" t="inlineStr">
         <is>
           <t>FILHET-ALLARD - Courtier assurance</t>
         </is>
@@ -2998,12 +3012,12 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="20" t="inlineStr">
+      <c r="A26" s="37" t="inlineStr">
         <is>
           <t>4010 0036</t>
         </is>
       </c>
-      <c r="B26" s="21" t="inlineStr">
+      <c r="B26" s="38" t="inlineStr">
         <is>
           <t>L'EAU D'ILE-DE-FRANCE</t>
         </is>
@@ -3037,12 +3051,12 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="20" t="inlineStr">
+      <c r="A27" s="37" t="inlineStr">
         <is>
           <t>4080 0001</t>
         </is>
       </c>
-      <c r="B27" s="21" t="inlineStr">
+      <c r="B27" s="38" t="inlineStr">
         <is>
           <t>Factures non parvenues</t>
         </is>
@@ -3076,12 +3090,12 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="20" t="inlineStr">
+      <c r="A28" s="37" t="inlineStr">
         <is>
           <t>4310 0001</t>
         </is>
       </c>
-      <c r="B28" s="21" t="inlineStr">
+      <c r="B28" s="38" t="inlineStr">
         <is>
           <t>URSSAF - Sécurité sociale</t>
         </is>
@@ -3115,12 +3129,12 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="20" t="inlineStr">
+      <c r="A29" s="37" t="inlineStr">
         <is>
           <t>4320 1002</t>
         </is>
       </c>
-      <c r="B29" s="21" t="inlineStr">
+      <c r="B29" s="38" t="inlineStr">
         <is>
           <t>HUMANIS PREVOYANCE - Organisme</t>
         </is>
@@ -3154,12 +3168,12 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="20" t="inlineStr">
+      <c r="A30" s="37" t="inlineStr">
         <is>
           <t>4320 3003</t>
         </is>
       </c>
-      <c r="B30" s="21" t="inlineStr">
+      <c r="B30" s="38" t="inlineStr">
         <is>
           <t>HUMANIS RETRAITE - Organisme retraite</t>
         </is>
@@ -3193,12 +3207,12 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="20" t="inlineStr">
+      <c r="A31" s="37" t="inlineStr">
         <is>
           <t>4630 0004</t>
         </is>
       </c>
-      <c r="B31" s="21" t="inlineStr">
+      <c r="B31" s="38" t="inlineStr">
         <is>
           <t>Azzopardi - Ancien copropriétaire</t>
         </is>
@@ -3232,12 +3246,12 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="20" t="inlineStr">
+      <c r="A32" s="37" t="inlineStr">
         <is>
           <t>4711 0001</t>
         </is>
       </c>
-      <c r="B32" s="21" t="inlineStr">
+      <c r="B32" s="38" t="inlineStr">
         <is>
           <t>Régularisation des charges - Débiteur</t>
         </is>
@@ -3271,12 +3285,12 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="20" t="inlineStr">
+      <c r="A33" s="37" t="inlineStr">
         <is>
           <t>4712 0001</t>
         </is>
       </c>
-      <c r="B33" s="21" t="inlineStr">
+      <c r="B33" s="38" t="inlineStr">
         <is>
           <t>Régularisation des travaux - Débiteur - AG 2018</t>
         </is>
@@ -3310,12 +3324,12 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="20" t="inlineStr">
+      <c r="A34" s="37" t="inlineStr">
         <is>
           <t>4712 0002</t>
         </is>
       </c>
-      <c r="B34" s="21" t="inlineStr">
+      <c r="B34" s="38" t="inlineStr">
         <is>
           <t>Régularisation des travaux - Débiteur - AG 19/</t>
         </is>
@@ -3349,12 +3363,12 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="20" t="inlineStr">
+      <c r="A35" s="37" t="inlineStr">
         <is>
           <t>4721 0001</t>
         </is>
       </c>
-      <c r="B35" s="21" t="inlineStr">
+      <c r="B35" s="38" t="inlineStr">
         <is>
           <t>Régularisation des charges - Créditeur</t>
         </is>
@@ -3388,12 +3402,12 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="20" t="inlineStr">
+      <c r="A36" s="37" t="inlineStr">
         <is>
           <t>4722 0001</t>
         </is>
       </c>
-      <c r="B36" s="21" t="inlineStr">
+      <c r="B36" s="38" t="inlineStr">
         <is>
           <t>Régularisation des travaux - Créditeur - AG 2018</t>
         </is>
@@ -3427,12 +3441,12 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="20" t="inlineStr">
+      <c r="A37" s="37" t="inlineStr">
         <is>
           <t>4730 0000</t>
         </is>
       </c>
-      <c r="B37" s="21" t="inlineStr">
+      <c r="B37" s="38" t="inlineStr">
         <is>
           <t>Rompus</t>
         </is>
@@ -3466,12 +3480,12 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="20" t="inlineStr">
+      <c r="A38" s="37" t="inlineStr">
         <is>
           <t>5120 0001</t>
         </is>
       </c>
-      <c r="B38" s="21" t="inlineStr">
+      <c r="B38" s="38" t="inlineStr">
         <is>
           <t>Compte courant Montepaschi - SDC DU 17 RUE</t>
         </is>
@@ -3505,12 +3519,12 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="20" t="inlineStr">
+      <c r="A39" s="37" t="inlineStr">
         <is>
           <t>5120 0004</t>
         </is>
       </c>
-      <c r="B39" s="21" t="inlineStr">
+      <c r="B39" s="38" t="inlineStr">
         <is>
           <t>Livret A Monte Paschi - LIVRET A 17 RUE LEON</t>
         </is>
@@ -3544,12 +3558,12 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="20" t="inlineStr">
+      <c r="A40" s="37" t="inlineStr">
         <is>
           <t>6010 0001</t>
         </is>
       </c>
-      <c r="B40" s="21" t="inlineStr">
+      <c r="B40" s="38" t="inlineStr">
         <is>
           <t>Facture d'eau</t>
         </is>
@@ -3583,12 +3597,12 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="20" t="inlineStr">
+      <c r="A41" s="37" t="inlineStr">
         <is>
           <t>6020 0001</t>
         </is>
       </c>
-      <c r="B41" s="21" t="inlineStr">
+      <c r="B41" s="38" t="inlineStr">
         <is>
           <t>Consommation Électricité</t>
         </is>
@@ -3622,12 +3636,12 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="20" t="inlineStr">
+      <c r="A42" s="37" t="inlineStr">
         <is>
           <t>6110 0001</t>
         </is>
       </c>
-      <c r="B42" s="21" t="inlineStr">
+      <c r="B42" s="38" t="inlineStr">
         <is>
           <t>Entretien nettoyage</t>
         </is>
@@ -3661,12 +3675,12 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="20" t="inlineStr">
+      <c r="A43" s="37" t="inlineStr">
         <is>
           <t>6140 0015</t>
         </is>
       </c>
-      <c r="B43" s="21" t="inlineStr">
+      <c r="B43" s="38" t="inlineStr">
         <is>
           <t>Entretien divers</t>
         </is>
@@ -3700,12 +3714,12 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="20" t="inlineStr">
+      <c r="A44" s="37" t="inlineStr">
         <is>
           <t>6140 0018</t>
         </is>
       </c>
-      <c r="B44" s="21" t="inlineStr">
+      <c r="B44" s="38" t="inlineStr">
         <is>
           <t>Contrat entretien - Jardins &amp; espaces verts</t>
         </is>
@@ -3739,12 +3753,12 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="20" t="inlineStr">
+      <c r="A45" s="37" t="inlineStr">
         <is>
           <t>6140 0019</t>
         </is>
       </c>
-      <c r="B45" s="21" t="inlineStr">
+      <c r="B45" s="38" t="inlineStr">
         <is>
           <t>Contrat service informatique</t>
         </is>
@@ -3778,12 +3792,12 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="20" t="inlineStr">
+      <c r="A46" s="37" t="inlineStr">
         <is>
           <t>6140 0023</t>
         </is>
       </c>
-      <c r="B46" s="21" t="inlineStr">
+      <c r="B46" s="38" t="inlineStr">
         <is>
           <t>Contrat de sécurité incendie</t>
         </is>
@@ -3817,12 +3831,12 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="20" t="inlineStr">
+      <c r="A47" s="37" t="inlineStr">
         <is>
           <t>6150 0030</t>
         </is>
       </c>
-      <c r="B47" s="21" t="inlineStr">
+      <c r="B47" s="38" t="inlineStr">
         <is>
           <t>Travaux divers</t>
         </is>
@@ -3856,12 +3870,12 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="20" t="inlineStr">
+      <c r="A48" s="37" t="inlineStr">
         <is>
           <t>6160 0001</t>
         </is>
       </c>
-      <c r="B48" s="21" t="inlineStr">
+      <c r="B48" s="38" t="inlineStr">
         <is>
           <t>Assurance multi-risques</t>
         </is>
@@ -3895,12 +3909,12 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="20" t="inlineStr">
+      <c r="A49" s="37" t="inlineStr">
         <is>
           <t>6160 0003</t>
         </is>
       </c>
-      <c r="B49" s="21" t="inlineStr">
+      <c r="B49" s="38" t="inlineStr">
         <is>
           <t>Protection juridique</t>
         </is>
@@ -3934,12 +3948,12 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="20" t="inlineStr">
+      <c r="A50" s="37" t="inlineStr">
         <is>
           <t>6211 0001</t>
         </is>
       </c>
-      <c r="B50" s="21" t="inlineStr">
+      <c r="B50" s="38" t="inlineStr">
         <is>
           <t>Honoraires gestion syndic</t>
         </is>
@@ -3973,12 +3987,12 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="20" t="inlineStr">
+      <c r="A51" s="37" t="inlineStr">
         <is>
           <t>6213 0001</t>
         </is>
       </c>
-      <c r="B51" s="21" t="inlineStr">
+      <c r="B51" s="38" t="inlineStr">
         <is>
           <t>Frais d'acheminement</t>
         </is>
@@ -4012,12 +4026,12 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="20" t="inlineStr">
+      <c r="A52" s="37" t="inlineStr">
         <is>
           <t>6213 0002</t>
         </is>
       </c>
-      <c r="B52" s="21" t="inlineStr">
+      <c r="B52" s="38" t="inlineStr">
         <is>
           <t>Affranchissements</t>
         </is>
@@ -4051,12 +4065,12 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="20" t="inlineStr">
+      <c r="A53" s="37" t="inlineStr">
         <is>
           <t>6221 0201</t>
         </is>
       </c>
-      <c r="B53" s="21" t="inlineStr">
+      <c r="B53" s="38" t="inlineStr">
         <is>
           <t>AG 19/07/23 Réso 22 Installation d'une haie -</t>
         </is>
@@ -4090,12 +4104,12 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="20" t="inlineStr">
+      <c r="A54" s="37" t="inlineStr">
         <is>
           <t>6222 0001</t>
         </is>
       </c>
-      <c r="B54" s="21" t="inlineStr">
+      <c r="B54" s="38" t="inlineStr">
         <is>
           <t>Vacations complémentaires</t>
         </is>
@@ -4129,12 +4143,12 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="20" t="inlineStr">
+      <c r="A55" s="37" t="inlineStr">
         <is>
           <t>6222 0002</t>
         </is>
       </c>
-      <c r="B55" s="21" t="inlineStr">
+      <c r="B55" s="38" t="inlineStr">
         <is>
           <t>Réunions CS &amp; AG complémentaires</t>
         </is>
@@ -4168,12 +4182,12 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="20" t="inlineStr">
+      <c r="A56" s="37" t="inlineStr">
         <is>
           <t>6222 0005</t>
         </is>
       </c>
-      <c r="B56" s="21" t="inlineStr">
+      <c r="B56" s="38" t="inlineStr">
         <is>
           <t>Pilotage et suivi des contentieux</t>
         </is>
@@ -4207,12 +4221,12 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="20" t="inlineStr">
+      <c r="A57" s="37" t="inlineStr">
         <is>
           <t>6222 0006</t>
         </is>
       </c>
-      <c r="B57" s="21" t="inlineStr">
+      <c r="B57" s="38" t="inlineStr">
         <is>
           <t>Frais de recouvrement</t>
         </is>
@@ -4246,12 +4260,12 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="20" t="inlineStr">
+      <c r="A58" s="37" t="inlineStr">
         <is>
           <t>6222 0007</t>
         </is>
       </c>
-      <c r="B58" s="21" t="inlineStr">
+      <c r="B58" s="38" t="inlineStr">
         <is>
           <t>Frais et honoraires liés aux mutations</t>
         </is>
@@ -4285,12 +4299,12 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="20" t="inlineStr">
+      <c r="A59" s="37" t="inlineStr">
         <is>
           <t>6230 0002</t>
         </is>
       </c>
-      <c r="B59" s="21" t="inlineStr">
+      <c r="B59" s="38" t="inlineStr">
         <is>
           <t>Honoraires huissiers</t>
         </is>
@@ -4324,12 +4338,12 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="20" t="inlineStr">
+      <c r="A60" s="37" t="inlineStr">
         <is>
           <t>6230 0003</t>
         </is>
       </c>
-      <c r="B60" s="21" t="inlineStr">
+      <c r="B60" s="38" t="inlineStr">
         <is>
           <t>Honoraires avocats</t>
         </is>
@@ -4363,12 +4377,12 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="20" t="inlineStr">
+      <c r="A61" s="37" t="inlineStr">
         <is>
           <t>6620 0001</t>
         </is>
       </c>
-      <c r="B61" s="21" t="inlineStr">
+      <c r="B61" s="38" t="inlineStr">
         <is>
           <t>Frais bancaires</t>
         </is>
@@ -4402,12 +4416,12 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="20" t="inlineStr">
+      <c r="A62" s="37" t="inlineStr">
         <is>
           <t>6620 0002</t>
         </is>
       </c>
-      <c r="B62" s="21" t="inlineStr">
+      <c r="B62" s="38" t="inlineStr">
         <is>
           <t>Reliquat de répartition</t>
         </is>
@@ -4441,12 +4455,12 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="20" t="inlineStr">
+      <c r="A63" s="37" t="inlineStr">
         <is>
           <t>6710 0201</t>
         </is>
       </c>
-      <c r="B63" s="21" t="inlineStr">
+      <c r="B63" s="38" t="inlineStr">
         <is>
           <t>AG 19/07/23 Réso 22 Installation d'une haie -</t>
         </is>
@@ -4480,12 +4494,12 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="20" t="inlineStr">
+      <c r="A64" s="37" t="inlineStr">
         <is>
           <t>6780 0003</t>
         </is>
       </c>
-      <c r="B64" s="21" t="inlineStr">
+      <c r="B64" s="38" t="inlineStr">
         <is>
           <t>Charges exceptionnelles sur exercices</t>
         </is>
@@ -4519,12 +4533,12 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="20" t="inlineStr">
+      <c r="A65" s="37" t="inlineStr">
         <is>
           <t>6900 0000</t>
         </is>
       </c>
-      <c r="B65" s="21" t="inlineStr">
+      <c r="B65" s="38" t="inlineStr">
         <is>
           <t>Charges et frais privatifs</t>
         </is>
@@ -4558,12 +4572,12 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="20" t="inlineStr">
+      <c r="A66" s="37" t="inlineStr">
         <is>
           <t>7010 0001</t>
         </is>
       </c>
-      <c r="B66" s="21" t="inlineStr">
+      <c r="B66" s="38" t="inlineStr">
         <is>
           <t>Provisions sur opérations courantes</t>
         </is>
@@ -4597,12 +4611,12 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="20" t="inlineStr">
+      <c r="A67" s="37" t="inlineStr">
         <is>
           <t>7180 0000</t>
         </is>
       </c>
-      <c r="B67" s="21" t="inlineStr">
+      <c r="B67" s="38" t="inlineStr">
         <is>
           <t>Produits exceptionnels</t>
         </is>

</xml_diff>

<commit_message>
Intégration données Matera (nouveau syndic) pour 2025 complet
- Parser CSV Matera avec neutralisation des reprises de l'ancien syndic
  (Solde antérieur, Dépensé avant le 28/07/2025, Transferts fonds travaux)
- Fusion MANDA (01/01-20/07) + Matera (28/07-31/12) pour l'exercice 2025
- Mapping des comptes Matera vers le plan comptable existant
- Nouveaux postes : Matera syndic (6140), Taxe foncière (6330),
  Frais CS/AG (6240), Intérêts livret A (7050)
- Bilan 2025 : soldes finaux issus du CSV Matera, équilibré
- Résultats : 2023=-786€ / 2024=+7511€ / 2025=+7618€ (CR détaillé)

Co-authored-by: alainannickbaptiste-dot <alainannickbaptiste-dot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/bilan_comptable_comparatif.xlsx
+++ b/bilan_comptable_comparatif.xlsx
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -700,7 +700,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Basé sur les mouvements de l'exercice (hors à-nouveaux, clôtures et décomptes)</t>
+          <t>Basé sur les mouvements de l'exercice (2025 = MANDA + Matera, reprises ancien syndic neutralisées)</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       <c r="D5" s="4" t="inlineStr">
         <is>
           <t>2025
-(01/01 - 20/07)*</t>
+(01/01 - 31/12)*</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
         <v>1018.55</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>267.62</v>
+        <v>758.85</v>
       </c>
     </row>
     <row r="8">
@@ -768,7 +768,7 @@
         <v>427.04</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>2.349999999999994</v>
+        <v>1191.48</v>
       </c>
     </row>
     <row r="9">
@@ -784,7 +784,7 @@
         <v>1445.59</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>269.97</v>
+        <v>1950.33</v>
       </c>
     </row>
     <row r="11">
@@ -874,158 +874,158 @@
         <v>362.35</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>0</v>
+        <v>230.63</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6150 0030 - Travaux divers</t>
+          <t xml:space="preserve">   6140 0036 - Abonnement Matera (syndic)</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>1411.66</v>
+        <v>0</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>1281.5</v>
+        <v>0</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>0</v>
+        <v>1457.99</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6160 0001 - Assurance multi-risques</t>
+          <t xml:space="preserve">   6150 0030 - Travaux divers</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>939.8200000000001</v>
+        <v>1411.66</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>948.46</v>
+        <v>1281.5</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>998.97</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">   6160 0001 - Assurance multi-risques</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>939.8200000000001</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>948.46</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>998.97</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">   6160 0003 - Protection juridique</t>
         </is>
       </c>
-      <c r="B19" s="7" t="n">
+      <c r="B20" s="7" t="n">
         <v>138</v>
       </c>
-      <c r="C19" s="7" t="n">
+      <c r="C20" s="7" t="n">
         <v>138</v>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D20" s="7" t="n">
         <v>-138</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Sous-total 61 - SERVICES EXTÉRIEURS</t>
         </is>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B21" s="9" t="n">
         <v>4726.55</v>
       </c>
-      <c r="C20" s="9" t="n">
+      <c r="C21" s="9" t="n">
         <v>4186.25</v>
       </c>
-      <c r="D20" s="9" t="n">
-        <v>890.72</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="D21" s="9" t="n">
+        <v>2579.34</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>62 - AUTRES SERVICES EXTÉRIEURS</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   6211 0001 - Honoraires gestion syndic</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="n">
-        <v>1800</v>
-      </c>
-      <c r="C23" s="7" t="n">
-        <v>1800</v>
-      </c>
-      <c r="D23" s="7" t="n">
-        <v>900</v>
-      </c>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6213 0001 - Frais d'acheminement</t>
+          <t xml:space="preserve">   6211 0001 - Honoraires gestion syndic</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>0</v>
+        <v>1800</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>10.99</v>
+        <v>1800</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6213 0002 - Affranchissements</t>
+          <t xml:space="preserve">   6213 0001 - Frais d'acheminement</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>82.11</v>
+        <v>0</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>62.41</v>
+        <v>10.99</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>26.38</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6221 0201 - AG 19/07/23 Réso 22 Installation d'une haie -</t>
+          <t xml:space="preserve">   6213 0002 - Affranchissements</t>
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>120</v>
+        <v>82.11</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>0</v>
+        <v>62.41</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>0</v>
+        <v>34.77</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6222 0001 - Vacations complémentaires</t>
+          <t xml:space="preserve">   6221 0201 - AG 19/07/23 Réso 22 Installation d'une haie -</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="D27" s="7" t="n">
         <v>0</v>
@@ -1034,14 +1034,14 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6222 0002 - Réunions CS &amp; AG complémentaires</t>
+          <t xml:space="preserve">   6222 0001 - Vacations complémentaires</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>240</v>
+        <v>0</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="D28" s="7" t="n">
         <v>0</v>
@@ -1050,11 +1050,11 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6222 0005 - Pilotage et suivi des contentieux</t>
+          <t xml:space="preserve">   6222 0002 - Réunions CS &amp; AG complémentaires</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>1668</v>
+        <v>240</v>
       </c>
       <c r="C29" s="7" t="n">
         <v>0</v>
@@ -1066,11 +1066,11 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6230 0002 - Honoraires huissiers</t>
+          <t xml:space="preserve">   6222 0005 - Pilotage et suivi des contentieux</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>495.4</v>
+        <v>1668</v>
       </c>
       <c r="C30" s="7" t="n">
         <v>0</v>
@@ -1082,338 +1082,444 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">   6230 0002 - Honoraires huissiers</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>495.4</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">   6230 0003 - Honoraires avocats</t>
         </is>
       </c>
-      <c r="B31" s="7" t="n">
+      <c r="B32" s="7" t="n">
         <v>4500.08</v>
       </c>
-      <c r="C31" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="C32" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   6230 0004 - Protection juridique (Filhet)</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>-278.48</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   6240 0001 - Frais du conseil syndical / AG</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>13.74</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>Sous-total 62 - AUTRES SERVICES EXTÉRIEURS</t>
         </is>
       </c>
-      <c r="B32" s="9" t="n">
+      <c r="B35" s="9" t="n">
         <v>8905.59</v>
       </c>
-      <c r="C32" s="9" t="n">
+      <c r="C35" s="9" t="n">
         <v>1969.4</v>
       </c>
-      <c r="D32" s="9" t="n">
-        <v>926.38</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="D35" s="9" t="n">
+        <v>670.03</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>63 - AUTRES</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n"/>
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   6330 0001 - Taxe foncière</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sous-total 63 - </t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="9" t="n">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>66 - CHARGES FINANCIÈRES</t>
         </is>
       </c>
-      <c r="B34" s="5" t="n"/>
-      <c r="C34" s="5" t="n"/>
-      <c r="D34" s="5" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="B41" s="5" t="n"/>
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="5" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   6620 0001 - Frais bancaires</t>
         </is>
       </c>
-      <c r="B35" s="7" t="n">
+      <c r="B42" s="7" t="n">
         <v>286.54</v>
       </c>
-      <c r="C35" s="7" t="n">
+      <c r="C42" s="7" t="n">
         <v>96</v>
       </c>
-      <c r="D35" s="7" t="n">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
+      <c r="D42" s="7" t="n">
+        <v>170.4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   6620 0002 - Reliquat de répartition</t>
         </is>
       </c>
-      <c r="B36" s="7" t="n">
+      <c r="B43" s="7" t="n">
         <v>0.25</v>
       </c>
-      <c r="C36" s="7" t="n">
+      <c r="C43" s="7" t="n">
         <v>0.06</v>
       </c>
-      <c r="D36" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="D43" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>Sous-total 66 - CHARGES FINANCIÈRES</t>
         </is>
       </c>
-      <c r="B37" s="9" t="n">
+      <c r="B44" s="9" t="n">
         <v>286.79</v>
       </c>
-      <c r="C37" s="9" t="n">
+      <c r="C44" s="9" t="n">
         <v>96.06</v>
       </c>
-      <c r="D37" s="9" t="n">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="D44" s="9" t="n">
+        <v>170.4</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>67 - CHARGES EXCEPTIONNELLES / TRAVAUX AG</t>
         </is>
       </c>
-      <c r="B39" s="5" t="n"/>
-      <c r="C39" s="5" t="n"/>
-      <c r="D39" s="5" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="B46" s="5" t="n"/>
+      <c r="C46" s="5" t="n"/>
+      <c r="D46" s="5" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   6710 0201 - AG 19/07/23 Réso 22 Installation d'une haie -</t>
         </is>
       </c>
-      <c r="B40" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C40" s="7" t="n">
+      <c r="B47" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="7" t="n">
         <v>792</v>
       </c>
-      <c r="D40" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
+      <c r="D47" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   6780 0003 - Charges exceptionnelles sur exercices</t>
         </is>
       </c>
-      <c r="B41" s="7" t="n">
+      <c r="B48" s="7" t="n">
         <v>25.49</v>
       </c>
-      <c r="C41" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D41" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="C48" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>Sous-total 67 - CHARGES EXCEPTIONNELLES / TRAVAUX AG</t>
         </is>
       </c>
-      <c r="B42" s="9" t="n">
+      <c r="B49" s="9" t="n">
         <v>25.49</v>
       </c>
-      <c r="C42" s="9" t="n">
+      <c r="C49" s="9" t="n">
         <v>792</v>
       </c>
-      <c r="D42" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="10" t="inlineStr">
+      <c r="D49" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
         <is>
           <t>TOTAL CHARGES (Classe 6)</t>
         </is>
       </c>
-      <c r="B44" s="11" t="n">
+      <c r="B51" s="11" t="n">
         <v>19186.03</v>
       </c>
-      <c r="C44" s="11" t="n">
+      <c r="C51" s="11" t="n">
         <v>8489.299999999999</v>
       </c>
-      <c r="D44" s="11" t="n">
-        <v>2159.07</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+      <c r="D51" s="11" t="n">
+        <v>6109.1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>PRODUITS (Classe 7)</t>
         </is>
       </c>
-      <c r="B47" s="4" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="D54" s="4" t="inlineStr">
         <is>
           <t>2025*</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>70 - PROVISIONS SUR CHARGES</t>
         </is>
       </c>
-      <c r="B48" s="5" t="n"/>
-      <c r="C48" s="5" t="n"/>
-      <c r="D48" s="5" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
+      <c r="B55" s="5" t="n"/>
+      <c r="C55" s="5" t="n"/>
+      <c r="D55" s="5" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   7010 0001 - Provisions sur opérations courantes</t>
         </is>
       </c>
-      <c r="B49" s="7" t="n">
+      <c r="B56" s="7" t="n">
         <v>18000</v>
       </c>
-      <c r="C49" s="7" t="n">
+      <c r="C56" s="7" t="n">
         <v>16000</v>
       </c>
-      <c r="D49" s="7" t="n">
-        <v>10274.94</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="D56" s="7" t="n">
+        <v>13700</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   7050 0001 - Intérêts livret A</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" s="7" t="n">
+        <v>27.44</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>Sous-total 70 - PROVISIONS SUR CHARGES</t>
         </is>
       </c>
-      <c r="B50" s="9" t="n">
+      <c r="B58" s="9" t="n">
         <v>18000</v>
       </c>
-      <c r="C50" s="9" t="n">
+      <c r="C58" s="9" t="n">
         <v>16000</v>
       </c>
-      <c r="D50" s="9" t="n">
-        <v>10274.94</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="D58" s="9" t="n">
+        <v>13727.44</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>71 - PRODUITS EXCEPTIONNELS</t>
         </is>
       </c>
-      <c r="B52" s="5" t="n"/>
-      <c r="C52" s="5" t="n"/>
-      <c r="D52" s="5" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="inlineStr">
+      <c r="B60" s="5" t="n"/>
+      <c r="C60" s="5" t="n"/>
+      <c r="D60" s="5" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   7180 0000 - Produits exceptionnels</t>
         </is>
       </c>
-      <c r="B53" s="7" t="n">
+      <c r="B61" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="C53" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D53" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="C61" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D61" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
         <is>
           <t>Sous-total 71 - PRODUITS EXCEPTIONNELS</t>
         </is>
       </c>
-      <c r="B54" s="9" t="n">
+      <c r="B62" s="9" t="n">
         <v>400</v>
       </c>
-      <c r="C54" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="12" t="inlineStr">
+      <c r="C62" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D62" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
         <is>
           <t>TOTAL PRODUITS (Classe 7)</t>
         </is>
       </c>
-      <c r="B56" s="13" t="n">
+      <c r="B64" s="13" t="n">
         <v>18400</v>
       </c>
-      <c r="C56" s="13" t="n">
+      <c r="C64" s="13" t="n">
         <v>16000</v>
       </c>
-      <c r="D56" s="13" t="n">
-        <v>10274.94</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="4" t="inlineStr">
+      <c r="D64" s="13" t="n">
+        <v>13727.44</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
         <is>
           <t>RÉSULTAT DE L'EXERCICE</t>
         </is>
       </c>
-      <c r="B59" s="4" t="inlineStr">
+      <c r="B67" s="4" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C67" s="4" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr">
+      <c r="D67" s="4" t="inlineStr">
         <is>
           <t>2025*</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="14" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
         <is>
           <t>Résultat = Produits - Charges</t>
         </is>
       </c>
-      <c r="B60" s="15" t="n">
+      <c r="B68" s="15" t="n">
         <v>-786.0299999999988</v>
       </c>
-      <c r="C60" s="15" t="n">
+      <c r="C68" s="15" t="n">
         <v>7510.700000000001</v>
       </c>
-      <c r="D60" s="15" t="n">
-        <v>8115.870000000001</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="16" t="inlineStr">
+      <c r="D68" s="15" t="n">
+        <v>7618.34</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="16" t="inlineStr">
         <is>
           <t>Résultat positif = excédent | Résultat négatif = déficit</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="17" t="inlineStr">
-        <is>
-          <t>* 2025 : exercice en cours au 20/07/2025, données partielles.</t>
+    <row r="71">
+      <c r="A71" s="17" t="inlineStr">
+        <is>
+          <t>* 2025 : exercice en cours (MANDA 01/01-20/07 + Matera 28/07-31/12). Reprises de l'ancien syndic neutralisées.</t>
         </is>
       </c>
     </row>
@@ -1582,7 +1688,7 @@
         <v>1742.55</v>
       </c>
       <c r="I7" s="26" t="n">
-        <v>2256.18</v>
+        <v>2427.54</v>
       </c>
     </row>
     <row r="8">
@@ -1607,7 +1713,7 @@
         <v>3742.55</v>
       </c>
       <c r="I8" s="30" t="n">
-        <v>4256.18</v>
+        <v>4427.54</v>
       </c>
     </row>
     <row r="9">
@@ -1623,7 +1729,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="26" t="n">
-        <v>3776.31</v>
+        <v>921.87</v>
       </c>
       <c r="E9" s="21" t="n"/>
       <c r="F9" s="24" t="inlineStr">
@@ -1648,7 +1754,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="28" t="n">
-        <v>3776.31</v>
+        <v>921.87</v>
       </c>
       <c r="E10" s="21" t="n"/>
       <c r="F10" s="25" t="inlineStr">
@@ -1704,7 +1810,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="26" t="n">
-        <v>278.48</v>
+        <v>11.74</v>
       </c>
       <c r="E12" s="21" t="n"/>
       <c r="F12" s="29" t="inlineStr">
@@ -1735,7 +1841,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>278.48</v>
+        <v>11.74</v>
       </c>
       <c r="E13" s="21" t="n"/>
       <c r="F13" s="24" t="inlineStr">
@@ -1775,7 +1881,7 @@
     <row r="15">
       <c r="A15" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Régularisation charges débiteur (4711)</t>
+          <t xml:space="preserve">   Régularisation charges débiteur (471)</t>
         </is>
       </c>
       <c r="B15" s="26" t="n">
@@ -1785,7 +1891,7 @@
         <v>26363.21</v>
       </c>
       <c r="D15" s="26" t="n">
-        <v>26363.21</v>
+        <v>26362.57</v>
       </c>
       <c r="E15" s="21" t="n"/>
       <c r="F15" s="29" t="inlineStr">
@@ -1816,7 +1922,7 @@
         <v>911.97</v>
       </c>
       <c r="D16" s="26" t="n">
-        <v>911.97</v>
+        <v>0</v>
       </c>
       <c r="E16" s="21" t="n"/>
       <c r="F16" s="24" t="inlineStr">
@@ -1841,12 +1947,12 @@
         <v>0.09</v>
       </c>
       <c r="D17" s="26" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="E17" s="21" t="n"/>
       <c r="F17" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Régularisation charges créditeur (4721)</t>
+          <t xml:space="preserve">   Régularisation charges créditeur (472)</t>
         </is>
       </c>
       <c r="G17" s="26" t="n">
@@ -1872,22 +1978,22 @@
         <v>27275.27</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>27275.27</v>
+        <v>26362.57</v>
       </c>
       <c r="E18" s="21" t="n"/>
-      <c r="F18" s="29" t="inlineStr">
-        <is>
-          <t>Total Comptes de régularisation - Passif</t>
-        </is>
-      </c>
-      <c r="G18" s="30" t="n">
-        <v>18000</v>
-      </c>
-      <c r="H18" s="30" t="n">
-        <v>34000</v>
-      </c>
-      <c r="I18" s="30" t="n">
-        <v>34000</v>
+      <c r="F18" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Rompus (473)</t>
+        </is>
+      </c>
+      <c r="G18" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="26" t="n">
+        <v>0.16</v>
       </c>
     </row>
     <row r="19">
@@ -1900,15 +2006,25 @@
       <c r="C19" s="23" t="inlineStr"/>
       <c r="D19" s="23" t="inlineStr"/>
       <c r="E19" s="21" t="n"/>
-      <c r="F19" s="25" t="inlineStr"/>
-      <c r="G19" s="25" t="inlineStr"/>
-      <c r="H19" s="25" t="inlineStr"/>
-      <c r="I19" s="25" t="inlineStr"/>
+      <c r="F19" s="29" t="inlineStr">
+        <is>
+          <t>Total Comptes de régularisation - Passif</t>
+        </is>
+      </c>
+      <c r="G19" s="30" t="n">
+        <v>18000</v>
+      </c>
+      <c r="H19" s="30" t="n">
+        <v>34000</v>
+      </c>
+      <c r="I19" s="30" t="n">
+        <v>34000.16</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Compte courant Montepaschi</t>
+          <t xml:space="preserve">   Compte courant (512)</t>
         </is>
       </c>
       <c r="B20" s="26" t="n">
@@ -1918,7 +2034,7 @@
         <v>9525.9</v>
       </c>
       <c r="D20" s="26" t="n">
-        <v>13074.46</v>
+        <v>17837.17</v>
       </c>
       <c r="E20" s="21" t="n"/>
       <c r="F20" s="25" t="inlineStr"/>
@@ -1939,7 +2055,7 @@
         <v>1742.55</v>
       </c>
       <c r="D21" s="26" t="n">
-        <v>1967.53</v>
+        <v>0</v>
       </c>
       <c r="E21" s="21" t="n"/>
       <c r="F21" s="25" t="inlineStr"/>
@@ -1960,7 +2076,7 @@
         <v>11268.45</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>15041.99</v>
+        <v>17837.17</v>
       </c>
       <c r="E22" s="21" t="n"/>
       <c r="F22" s="25" t="inlineStr"/>
@@ -1986,7 +2102,7 @@
         <v>0</v>
       </c>
       <c r="I24" s="33" t="n">
-        <v>8115.870000000001</v>
+        <v>6705.649999999994</v>
       </c>
     </row>
     <row r="25">
@@ -2005,7 +2121,7 @@
         <v>38543.72</v>
       </c>
       <c r="D26" s="35" t="n">
-        <v>46372.05</v>
+        <v>45133.35</v>
       </c>
       <c r="E26" s="21" t="n"/>
       <c r="F26" s="34" t="inlineStr">
@@ -2020,7 +2136,7 @@
         <v>38543.72</v>
       </c>
       <c r="I26" s="35" t="n">
-        <v>46372.05</v>
+        <v>45133.35</v>
       </c>
     </row>
     <row r="28">
@@ -2047,7 +2163,7 @@
     <row r="32">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>* 2025 : exercice en cours au 20/07/2025 (non clôturé).</t>
+          <t>* 2025 : exercice en cours (MANDA 01/01-20/07 + Matera 28/07-31/12, reprises neutralisées).</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K67"/>
+  <dimension ref="A1:K76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2225,10 +2341,10 @@
         <v>0</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>513.63</v>
+        <v>685</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-513.63</v>
+        <v>-685</v>
       </c>
     </row>
     <row r="6">
@@ -2690,10 +2806,10 @@
         <v>0</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>144.07</v>
+        <v>1333.2</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>144.07</v>
+        <v>1333.2</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>0</v>
@@ -2768,10 +2884,10 @@
         <v>-362.35</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>362.35</v>
+        <v>592.98</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0</v>
+        <v>230.63</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>362.35</v>
@@ -3002,10 +3118,10 @@
         <v>0</v>
       </c>
       <c r="I25" s="7" t="n">
+        <v>697.4400000000001</v>
+      </c>
+      <c r="J25" s="7" t="n">
         <v>418.96</v>
-      </c>
-      <c r="J25" s="7" t="n">
-        <v>140.48</v>
       </c>
       <c r="K25" s="7" t="n">
         <v>278.48</v>
@@ -3041,10 +3157,10 @@
         <v>0</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>267.62</v>
+        <v>1973.15</v>
       </c>
       <c r="J26" s="7" t="n">
-        <v>267.62</v>
+        <v>1973.15</v>
       </c>
       <c r="K26" s="7" t="n">
         <v>0</v>
@@ -3053,61 +3169,61 @@
     <row r="27">
       <c r="A27" s="37" t="inlineStr">
         <is>
-          <t>4080 0001</t>
+          <t>4010 0037</t>
         </is>
       </c>
       <c r="B27" s="38" t="inlineStr">
         <is>
-          <t>Factures non parvenues</t>
+          <t>MySendingBox (Courriers)</t>
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>1609.92</v>
+        <v>0</v>
       </c>
       <c r="D27" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>1609.92</v>
+        <v>0</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>17699.99999999999</v>
+        <v>0</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>17841.72</v>
+        <v>0</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>-141.7200000000084</v>
+        <v>0</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>11550.29</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>7632.26</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>3918.029999999997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="37" t="inlineStr">
         <is>
-          <t>4310 0001</t>
+          <t>4010 0038</t>
         </is>
       </c>
       <c r="B28" s="38" t="inlineStr">
         <is>
-          <t>URSSAF - Sécurité sociale</t>
+          <t>DIRECTION GENERALE DES FINANCES PUBLIQUES</t>
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>619</v>
+        <v>0</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>1192</v>
+        <v>0</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>-573</v>
+        <v>0</v>
       </c>
       <c r="F28" s="7" t="n">
         <v>0</v>
@@ -3119,34 +3235,34 @@
         <v>0</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>0</v>
+        <v>486</v>
       </c>
       <c r="J28" s="7" t="n">
-        <v>0</v>
+        <v>739</v>
       </c>
       <c r="K28" s="7" t="n">
-        <v>0</v>
+        <v>-253</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="37" t="inlineStr">
         <is>
-          <t>4320 1002</t>
+          <t>4010 0039</t>
         </is>
       </c>
       <c r="B29" s="38" t="inlineStr">
         <is>
-          <t>HUMANIS PREVOYANCE - Organisme</t>
+          <t>AR24</t>
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>33.42</v>
+        <v>0</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>41.78</v>
+        <v>0</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>-8.359999999999999</v>
+        <v>0</v>
       </c>
       <c r="F29" s="7" t="n">
         <v>0</v>
@@ -3158,82 +3274,82 @@
         <v>0</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0</v>
+        <v>15.74</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>0</v>
+        <v>-13.74</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="37" t="inlineStr">
         <is>
-          <t>4320 3003</t>
+          <t>4080 0001</t>
         </is>
       </c>
       <c r="B30" s="38" t="inlineStr">
         <is>
-          <t>HUMANIS RETRAITE - Organisme retraite</t>
+          <t>Factures non parvenues</t>
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>24458.15000000001</v>
+        <v>1609.92</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>29311.38</v>
+        <v>0</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>-4853.229999999992</v>
+        <v>1609.92</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>0</v>
+        <v>17699.99999999999</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>0</v>
+        <v>17841.72</v>
       </c>
       <c r="H30" s="7" t="n">
-        <v>0</v>
+        <v>-141.7200000000084</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>0</v>
+        <v>11550.29</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>0</v>
+        <v>7632.26</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>0</v>
+        <v>3918.029999999997</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="37" t="inlineStr">
         <is>
-          <t>4630 0004</t>
+          <t>4310 0001</t>
         </is>
       </c>
       <c r="B31" s="38" t="inlineStr">
         <is>
-          <t>Azzopardi - Ancien copropriétaire</t>
+          <t>URSSAF - Sécurité sociale</t>
         </is>
       </c>
       <c r="C31" s="7" t="n">
-        <v>0</v>
+        <v>619</v>
       </c>
       <c r="D31" s="7" t="n">
-        <v>0</v>
+        <v>1192</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>0</v>
+        <v>-573</v>
       </c>
       <c r="F31" s="7" t="n">
-        <v>424</v>
+        <v>0</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>424</v>
+        <v>0</v>
       </c>
       <c r="I31" s="7" t="n">
         <v>0</v>
@@ -3248,22 +3364,22 @@
     <row r="32">
       <c r="A32" s="37" t="inlineStr">
         <is>
-          <t>4711 0001</t>
+          <t>4320 1002</t>
         </is>
       </c>
       <c r="B32" s="38" t="inlineStr">
         <is>
-          <t>Régularisation des charges - Débiteur</t>
+          <t>HUMANIS PREVOYANCE - Organisme</t>
         </is>
       </c>
       <c r="C32" s="7" t="n">
-        <v>0</v>
+        <v>33.42</v>
       </c>
       <c r="D32" s="7" t="n">
-        <v>57371.18</v>
+        <v>41.78</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>-57371.18</v>
+        <v>-8.359999999999999</v>
       </c>
       <c r="F32" s="7" t="n">
         <v>0</v>
@@ -3287,22 +3403,22 @@
     <row r="33">
       <c r="A33" s="37" t="inlineStr">
         <is>
-          <t>4712 0001</t>
+          <t>4320 3003</t>
         </is>
       </c>
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>Régularisation des travaux - Débiteur - AG 2018</t>
+          <t>HUMANIS RETRAITE - Organisme retraite</t>
         </is>
       </c>
       <c r="C33" s="7" t="n">
-        <v>0</v>
+        <v>24458.15000000001</v>
       </c>
       <c r="D33" s="7" t="n">
-        <v>3553.85</v>
+        <v>29311.38</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>-3553.85</v>
+        <v>-4853.229999999992</v>
       </c>
       <c r="F33" s="7" t="n">
         <v>0</v>
@@ -3326,12 +3442,12 @@
     <row r="34">
       <c r="A34" s="37" t="inlineStr">
         <is>
-          <t>4712 0002</t>
+          <t>450</t>
         </is>
       </c>
       <c r="B34" s="38" t="inlineStr">
         <is>
-          <t>Régularisation des travaux - Débiteur - AG 19/</t>
+          <t>Copropriétaires</t>
         </is>
       </c>
       <c r="C34" s="7" t="n">
@@ -3353,43 +3469,43 @@
         <v>0</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>0</v>
+        <v>3631.64</v>
       </c>
       <c r="J34" s="7" t="n">
-        <v>0</v>
+        <v>6665.959999999999</v>
       </c>
       <c r="K34" s="7" t="n">
-        <v>0</v>
+        <v>-3034.319999999999</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="37" t="inlineStr">
         <is>
-          <t>4721 0001</t>
+          <t>4630 0004</t>
         </is>
       </c>
       <c r="B35" s="38" t="inlineStr">
         <is>
-          <t>Régularisation des charges - Créditeur</t>
+          <t>Azzopardi - Ancien copropriétaire</t>
         </is>
       </c>
       <c r="C35" s="7" t="n">
-        <v>54000</v>
+        <v>0</v>
       </c>
       <c r="D35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>54000</v>
+        <v>0</v>
       </c>
       <c r="F35" s="7" t="n">
-        <v>0</v>
+        <v>424</v>
       </c>
       <c r="G35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>0</v>
+        <v>424</v>
       </c>
       <c r="I35" s="7" t="n">
         <v>0</v>
@@ -3404,22 +3520,22 @@
     <row r="36">
       <c r="A36" s="37" t="inlineStr">
         <is>
-          <t>4722 0001</t>
+          <t>4711 0001</t>
         </is>
       </c>
       <c r="B36" s="38" t="inlineStr">
         <is>
-          <t>Régularisation des travaux - Créditeur - AG 2018</t>
+          <t>Régularisation des charges - Débiteur</t>
         </is>
       </c>
       <c r="C36" s="7" t="n">
-        <v>3553.88</v>
+        <v>0</v>
       </c>
       <c r="D36" s="7" t="n">
-        <v>0</v>
+        <v>57371.18</v>
       </c>
       <c r="E36" s="7" t="n">
-        <v>3553.88</v>
+        <v>-57371.18</v>
       </c>
       <c r="F36" s="7" t="n">
         <v>0</v>
@@ -3431,43 +3547,43 @@
         <v>0</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>0</v>
+        <v>27.44</v>
       </c>
       <c r="J36" s="7" t="n">
-        <v>0</v>
+        <v>14889.5</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>0</v>
+        <v>-14862.06</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="37" t="inlineStr">
         <is>
-          <t>4730 0000</t>
+          <t>4712 0001</t>
         </is>
       </c>
       <c r="B37" s="38" t="inlineStr">
         <is>
-          <t>Rompus</t>
+          <t>Régularisation des travaux - Débiteur - AG 2018</t>
         </is>
       </c>
       <c r="C37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D37" s="7" t="n">
-        <v>0.25</v>
+        <v>3553.85</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>-0.25</v>
+        <v>-3553.85</v>
       </c>
       <c r="F37" s="7" t="n">
         <v>0</v>
       </c>
       <c r="G37" s="7" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>-0.06</v>
+        <v>0</v>
       </c>
       <c r="I37" s="7" t="n">
         <v>0</v>
@@ -3482,343 +3598,343 @@
     <row r="38">
       <c r="A38" s="37" t="inlineStr">
         <is>
-          <t>5120 0001</t>
+          <t>4712 0002</t>
         </is>
       </c>
       <c r="B38" s="38" t="inlineStr">
         <is>
-          <t>Compte courant Montepaschi - SDC DU 17 RUE</t>
+          <t>Régularisation des travaux - Débiteur - AG 19/</t>
         </is>
       </c>
       <c r="C38" s="7" t="n">
-        <v>28923.34</v>
+        <v>0</v>
       </c>
       <c r="D38" s="7" t="n">
-        <v>28970.87000000001</v>
+        <v>0</v>
       </c>
       <c r="E38" s="7" t="n">
-        <v>-47.53000000000611</v>
+        <v>0</v>
       </c>
       <c r="F38" s="7" t="n">
-        <v>17700</v>
+        <v>0</v>
       </c>
       <c r="G38" s="7" t="n">
-        <v>11142.13</v>
+        <v>0</v>
       </c>
       <c r="H38" s="7" t="n">
-        <v>6557.870000000001</v>
+        <v>0</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>7542.259999999999</v>
+        <v>0</v>
       </c>
       <c r="J38" s="7" t="n">
-        <v>3993.7</v>
+        <v>0</v>
       </c>
       <c r="K38" s="7" t="n">
-        <v>3548.559999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="37" t="inlineStr">
         <is>
-          <t>5120 0004</t>
+          <t>4721 0001</t>
         </is>
       </c>
       <c r="B39" s="38" t="inlineStr">
         <is>
-          <t>Livret A Monte Paschi - LIVRET A 17 RUE LEON</t>
+          <t>Régularisation des charges - Créditeur</t>
         </is>
       </c>
       <c r="C39" s="7" t="n">
-        <v>910.22</v>
+        <v>54000</v>
       </c>
       <c r="D39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>910.22</v>
+        <v>54000</v>
       </c>
       <c r="F39" s="7" t="n">
-        <v>832.3299999999999</v>
+        <v>0</v>
       </c>
       <c r="G39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>832.3299999999999</v>
+        <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>224.98</v>
+        <v>0</v>
       </c>
       <c r="J39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K39" s="7" t="n">
-        <v>224.98</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="37" t="inlineStr">
         <is>
-          <t>6010 0001</t>
+          <t>4722 0001</t>
         </is>
       </c>
       <c r="B40" s="38" t="inlineStr">
         <is>
-          <t>Facture d'eau</t>
+          <t>Régularisation des travaux - Créditeur - AG 2018</t>
         </is>
       </c>
       <c r="C40" s="7" t="n">
-        <v>2059.18</v>
+        <v>3553.88</v>
       </c>
       <c r="D40" s="7" t="n">
-        <v>1029.59</v>
+        <v>0</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>1029.59</v>
+        <v>3553.88</v>
       </c>
       <c r="F40" s="7" t="n">
-        <v>2037.31</v>
+        <v>0</v>
       </c>
       <c r="G40" s="7" t="n">
-        <v>1018.76</v>
+        <v>0</v>
       </c>
       <c r="H40" s="7" t="n">
-        <v>1018.55</v>
+        <v>0</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>267.62</v>
+        <v>0</v>
       </c>
       <c r="J40" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K40" s="7" t="n">
-        <v>267.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="37" t="inlineStr">
         <is>
-          <t>6020 0001</t>
+          <t>4730 0000</t>
         </is>
       </c>
       <c r="B41" s="38" t="inlineStr">
         <is>
-          <t>Consommation Électricité</t>
+          <t>Rompus</t>
         </is>
       </c>
       <c r="C41" s="7" t="n">
-        <v>5421.940000000001</v>
+        <v>0</v>
       </c>
       <c r="D41" s="7" t="n">
-        <v>1209.92</v>
+        <v>0.25</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>4212.02</v>
+        <v>-0.25</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>427.04</v>
+        <v>0</v>
       </c>
       <c r="G41" s="7" t="n">
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>427.04</v>
+        <v>-0.06</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>144.07</v>
+        <v>0.05</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>141.72</v>
+        <v>0.26</v>
       </c>
       <c r="K41" s="7" t="n">
-        <v>2.349999999999994</v>
+        <v>-0.21</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="37" t="inlineStr">
         <is>
-          <t>6110 0001</t>
+          <t>5120 0001</t>
         </is>
       </c>
       <c r="B42" s="38" t="inlineStr">
         <is>
-          <t>Entretien nettoyage</t>
+          <t>Compte courant Montepaschi - SDC DU 17 RUE</t>
         </is>
       </c>
       <c r="C42" s="7" t="n">
-        <v>1864.5</v>
+        <v>28923.34</v>
       </c>
       <c r="D42" s="7" t="n">
-        <v>0</v>
+        <v>28970.87000000001</v>
       </c>
       <c r="E42" s="7" t="n">
-        <v>1864.5</v>
+        <v>-47.53000000000611</v>
       </c>
       <c r="F42" s="7" t="n">
-        <v>0</v>
+        <v>17700</v>
       </c>
       <c r="G42" s="7" t="n">
-        <v>0</v>
+        <v>11142.13</v>
       </c>
       <c r="H42" s="7" t="n">
-        <v>0</v>
+        <v>6557.870000000001</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>0</v>
+        <v>29035.11</v>
       </c>
       <c r="J42" s="7" t="n">
-        <v>0</v>
+        <v>7649.38</v>
       </c>
       <c r="K42" s="7" t="n">
-        <v>0</v>
+        <v>21385.73</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="37" t="inlineStr">
         <is>
-          <t>6140 0015</t>
+          <t>5120 0004</t>
         </is>
       </c>
       <c r="B43" s="38" t="inlineStr">
         <is>
-          <t>Entretien divers</t>
+          <t>Livret A Monte Paschi - LIVRET A 17 RUE LEON</t>
         </is>
       </c>
       <c r="C43" s="7" t="n">
-        <v>0</v>
+        <v>910.22</v>
       </c>
       <c r="D43" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>0</v>
+        <v>910.22</v>
       </c>
       <c r="F43" s="7" t="n">
-        <v>260.7</v>
+        <v>832.3299999999999</v>
       </c>
       <c r="G43" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>260.7</v>
+        <v>832.3299999999999</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>0</v>
+        <v>224.98</v>
       </c>
       <c r="J43" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K43" s="7" t="n">
-        <v>0</v>
+        <v>224.98</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="37" t="inlineStr">
         <is>
-          <t>6140 0018</t>
+          <t>6010 0001</t>
         </is>
       </c>
       <c r="B44" s="38" t="inlineStr">
         <is>
-          <t>Contrat entretien - Jardins &amp; espaces verts</t>
+          <t>Facture d'eau</t>
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>0</v>
+        <v>2059.18</v>
       </c>
       <c r="D44" s="7" t="n">
-        <v>0</v>
+        <v>1029.59</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>0</v>
+        <v>1029.59</v>
       </c>
       <c r="F44" s="7" t="n">
-        <v>1167</v>
+        <v>2037.31</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>0</v>
+        <v>1018.76</v>
       </c>
       <c r="H44" s="7" t="n">
-        <v>1167</v>
+        <v>1018.55</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>0</v>
+        <v>758.85</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>0</v>
+        <v>758.85</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="37" t="inlineStr">
         <is>
-          <t>6140 0019</t>
+          <t>6020 0001</t>
         </is>
       </c>
       <c r="B45" s="38" t="inlineStr">
         <is>
-          <t>Contrat service informatique</t>
+          <t>Consommation Électricité</t>
         </is>
       </c>
       <c r="C45" s="7" t="n">
-        <v>26.51</v>
+        <v>5421.940000000001</v>
       </c>
       <c r="D45" s="7" t="n">
-        <v>0</v>
+        <v>1209.92</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>26.51</v>
+        <v>4212.02</v>
       </c>
       <c r="F45" s="7" t="n">
-        <v>28.24</v>
+        <v>427.04</v>
       </c>
       <c r="G45" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>28.24</v>
+        <v>427.04</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>29.75</v>
+        <v>1333.2</v>
       </c>
       <c r="J45" s="7" t="n">
-        <v>0</v>
+        <v>141.72</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>29.75</v>
+        <v>1191.48</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="37" t="inlineStr">
         <is>
-          <t>6140 0023</t>
+          <t>6110 0001</t>
         </is>
       </c>
       <c r="B46" s="38" t="inlineStr">
         <is>
-          <t>Contrat de sécurité incendie</t>
+          <t>Entretien nettoyage</t>
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>346.06</v>
+        <v>1864.5</v>
       </c>
       <c r="D46" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>346.06</v>
+        <v>1864.5</v>
       </c>
       <c r="F46" s="7" t="n">
-        <v>362.35</v>
+        <v>0</v>
       </c>
       <c r="G46" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H46" s="7" t="n">
-        <v>362.35</v>
+        <v>0</v>
       </c>
       <c r="I46" s="7" t="n">
         <v>0</v>
@@ -3833,31 +3949,31 @@
     <row r="47">
       <c r="A47" s="37" t="inlineStr">
         <is>
-          <t>6150 0030</t>
+          <t>6140 0015</t>
         </is>
       </c>
       <c r="B47" s="38" t="inlineStr">
         <is>
-          <t>Travaux divers</t>
+          <t>Entretien divers</t>
         </is>
       </c>
       <c r="C47" s="7" t="n">
-        <v>1411.66</v>
+        <v>0</v>
       </c>
       <c r="D47" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>1411.66</v>
+        <v>0</v>
       </c>
       <c r="F47" s="7" t="n">
-        <v>1281.5</v>
+        <v>260.7</v>
       </c>
       <c r="G47" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H47" s="7" t="n">
-        <v>1281.5</v>
+        <v>260.7</v>
       </c>
       <c r="I47" s="7" t="n">
         <v>0</v>
@@ -3872,129 +3988,129 @@
     <row r="48">
       <c r="A48" s="37" t="inlineStr">
         <is>
-          <t>6160 0001</t>
+          <t>6140 0018</t>
         </is>
       </c>
       <c r="B48" s="38" t="inlineStr">
         <is>
-          <t>Assurance multi-risques</t>
+          <t>Contrat entretien - Jardins &amp; espaces verts</t>
         </is>
       </c>
       <c r="C48" s="7" t="n">
-        <v>939.8200000000001</v>
+        <v>0</v>
       </c>
       <c r="D48" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E48" s="7" t="n">
-        <v>939.8200000000001</v>
+        <v>0</v>
       </c>
       <c r="F48" s="7" t="n">
-        <v>948.46</v>
+        <v>1167</v>
       </c>
       <c r="G48" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H48" s="7" t="n">
-        <v>948.46</v>
+        <v>1167</v>
       </c>
       <c r="I48" s="7" t="n">
-        <v>998.97</v>
+        <v>0</v>
       </c>
       <c r="J48" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K48" s="7" t="n">
-        <v>998.97</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="37" t="inlineStr">
         <is>
-          <t>6160 0003</t>
+          <t>6140 0019</t>
         </is>
       </c>
       <c r="B49" s="38" t="inlineStr">
         <is>
-          <t>Protection juridique</t>
+          <t>Contrat service informatique</t>
         </is>
       </c>
       <c r="C49" s="7" t="n">
-        <v>138</v>
+        <v>26.51</v>
       </c>
       <c r="D49" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>138</v>
+        <v>26.51</v>
       </c>
       <c r="F49" s="7" t="n">
-        <v>138</v>
+        <v>28.24</v>
       </c>
       <c r="G49" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H49" s="7" t="n">
-        <v>138</v>
+        <v>28.24</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>140.48</v>
+        <v>29.75</v>
       </c>
       <c r="J49" s="7" t="n">
-        <v>278.48</v>
+        <v>0</v>
       </c>
       <c r="K49" s="7" t="n">
-        <v>-138</v>
+        <v>29.75</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="37" t="inlineStr">
         <is>
-          <t>6211 0001</t>
+          <t>6140 0023</t>
         </is>
       </c>
       <c r="B50" s="38" t="inlineStr">
         <is>
-          <t>Honoraires gestion syndic</t>
+          <t>Contrat de sécurité incendie</t>
         </is>
       </c>
       <c r="C50" s="7" t="n">
-        <v>1800</v>
+        <v>346.06</v>
       </c>
       <c r="D50" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E50" s="7" t="n">
-        <v>1800</v>
+        <v>346.06</v>
       </c>
       <c r="F50" s="7" t="n">
-        <v>1800</v>
+        <v>362.35</v>
       </c>
       <c r="G50" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H50" s="7" t="n">
-        <v>1800</v>
+        <v>362.35</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>900</v>
+        <v>230.63</v>
       </c>
       <c r="J50" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>900</v>
+        <v>230.63</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="37" t="inlineStr">
         <is>
-          <t>6213 0001</t>
+          <t>6140 0036</t>
         </is>
       </c>
       <c r="B51" s="38" t="inlineStr">
         <is>
-          <t>Frais d'acheminement</t>
+          <t>Abonnement Matera (syndic)</t>
         </is>
       </c>
       <c r="C51" s="7" t="n">
@@ -4007,208 +4123,208 @@
         <v>0</v>
       </c>
       <c r="F51" s="7" t="n">
-        <v>10.99</v>
+        <v>0</v>
       </c>
       <c r="G51" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H51" s="7" t="n">
-        <v>10.99</v>
+        <v>0</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>0</v>
+        <v>1457.99</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>0</v>
+        <v>1457.99</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="37" t="inlineStr">
         <is>
-          <t>6213 0002</t>
+          <t>6150 0030</t>
         </is>
       </c>
       <c r="B52" s="38" t="inlineStr">
         <is>
-          <t>Affranchissements</t>
+          <t>Travaux divers</t>
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>82.11</v>
+        <v>1411.66</v>
       </c>
       <c r="D52" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E52" s="7" t="n">
-        <v>82.11</v>
+        <v>1411.66</v>
       </c>
       <c r="F52" s="7" t="n">
-        <v>62.41</v>
+        <v>1281.5</v>
       </c>
       <c r="G52" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H52" s="7" t="n">
-        <v>62.41</v>
+        <v>1281.5</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>26.38</v>
+        <v>0</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>26.38</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="37" t="inlineStr">
         <is>
-          <t>6221 0201</t>
+          <t>6160 0001</t>
         </is>
       </c>
       <c r="B53" s="38" t="inlineStr">
         <is>
-          <t>AG 19/07/23 Réso 22 Installation d'une haie -</t>
+          <t>Assurance multi-risques</t>
         </is>
       </c>
       <c r="C53" s="7" t="n">
-        <v>120</v>
+        <v>939.8200000000001</v>
       </c>
       <c r="D53" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>120</v>
+        <v>939.8200000000001</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>0</v>
+        <v>948.46</v>
       </c>
       <c r="G53" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H53" s="7" t="n">
-        <v>0</v>
+        <v>948.46</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>0</v>
+        <v>998.97</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0</v>
+        <v>998.97</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="37" t="inlineStr">
         <is>
-          <t>6222 0001</t>
+          <t>6160 0003</t>
         </is>
       </c>
       <c r="B54" s="38" t="inlineStr">
         <is>
-          <t>Vacations complémentaires</t>
+          <t>Protection juridique</t>
         </is>
       </c>
       <c r="C54" s="7" t="n">
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="D54" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E54" s="7" t="n">
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="F54" s="7" t="n">
-        <v>96</v>
+        <v>138</v>
       </c>
       <c r="G54" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H54" s="7" t="n">
-        <v>96</v>
+        <v>138</v>
       </c>
       <c r="I54" s="7" t="n">
-        <v>0</v>
+        <v>140.48</v>
       </c>
       <c r="J54" s="7" t="n">
-        <v>0</v>
+        <v>278.48</v>
       </c>
       <c r="K54" s="7" t="n">
-        <v>0</v>
+        <v>-138</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="37" t="inlineStr">
         <is>
-          <t>6222 0002</t>
+          <t>6211 0001</t>
         </is>
       </c>
       <c r="B55" s="38" t="inlineStr">
         <is>
-          <t>Réunions CS &amp; AG complémentaires</t>
+          <t>Honoraires gestion syndic</t>
         </is>
       </c>
       <c r="C55" s="7" t="n">
-        <v>240</v>
+        <v>1800</v>
       </c>
       <c r="D55" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>240</v>
+        <v>1800</v>
       </c>
       <c r="F55" s="7" t="n">
-        <v>0</v>
+        <v>1800</v>
       </c>
       <c r="G55" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H55" s="7" t="n">
-        <v>0</v>
+        <v>1800</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="J55" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K55" s="7" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="37" t="inlineStr">
         <is>
-          <t>6222 0005</t>
+          <t>6213 0001</t>
         </is>
       </c>
       <c r="B56" s="38" t="inlineStr">
         <is>
-          <t>Pilotage et suivi des contentieux</t>
+          <t>Frais d'acheminement</t>
         </is>
       </c>
       <c r="C56" s="7" t="n">
-        <v>1668</v>
+        <v>0</v>
       </c>
       <c r="D56" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E56" s="7" t="n">
-        <v>1668</v>
+        <v>0</v>
       </c>
       <c r="F56" s="7" t="n">
-        <v>0</v>
+        <v>10.99</v>
       </c>
       <c r="G56" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H56" s="7" t="n">
-        <v>0</v>
+        <v>10.99</v>
       </c>
       <c r="I56" s="7" t="n">
         <v>0</v>
@@ -4223,76 +4339,76 @@
     <row r="57">
       <c r="A57" s="37" t="inlineStr">
         <is>
-          <t>6222 0006</t>
+          <t>6213 0002</t>
         </is>
       </c>
       <c r="B57" s="38" t="inlineStr">
         <is>
-          <t>Frais de recouvrement</t>
+          <t>Affranchissements</t>
         </is>
       </c>
       <c r="C57" s="7" t="n">
-        <v>0</v>
+        <v>82.11</v>
       </c>
       <c r="D57" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E57" s="7" t="n">
-        <v>0</v>
+        <v>82.11</v>
       </c>
       <c r="F57" s="7" t="n">
-        <v>0</v>
+        <v>62.41</v>
       </c>
       <c r="G57" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H57" s="7" t="n">
-        <v>0</v>
+        <v>62.41</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>120</v>
+        <v>35.77</v>
       </c>
       <c r="J57" s="7" t="n">
-        <v>120</v>
+        <v>1</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0</v>
+        <v>34.77</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="37" t="inlineStr">
         <is>
-          <t>6222 0007</t>
+          <t>6221 0201</t>
         </is>
       </c>
       <c r="B58" s="38" t="inlineStr">
         <is>
-          <t>Frais et honoraires liés aux mutations</t>
+          <t>AG 19/07/23 Réso 22 Installation d'une haie -</t>
         </is>
       </c>
       <c r="C58" s="7" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E58" s="7" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="F58" s="7" t="n">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="G58" s="7" t="n">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="H58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I58" s="7" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="J58" s="7" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="K58" s="7" t="n">
         <v>0</v>
@@ -4301,31 +4417,31 @@
     <row r="59">
       <c r="A59" s="37" t="inlineStr">
         <is>
-          <t>6230 0002</t>
+          <t>6222 0001</t>
         </is>
       </c>
       <c r="B59" s="38" t="inlineStr">
         <is>
-          <t>Honoraires huissiers</t>
+          <t>Vacations complémentaires</t>
         </is>
       </c>
       <c r="C59" s="7" t="n">
-        <v>495.4</v>
+        <v>0</v>
       </c>
       <c r="D59" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E59" s="7" t="n">
-        <v>495.4</v>
+        <v>0</v>
       </c>
       <c r="F59" s="7" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="G59" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H59" s="7" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="I59" s="7" t="n">
         <v>0</v>
@@ -4340,22 +4456,22 @@
     <row r="60">
       <c r="A60" s="37" t="inlineStr">
         <is>
-          <t>6230 0003</t>
+          <t>6222 0002</t>
         </is>
       </c>
       <c r="B60" s="38" t="inlineStr">
         <is>
-          <t>Honoraires avocats</t>
+          <t>Réunions CS &amp; AG complémentaires</t>
         </is>
       </c>
       <c r="C60" s="7" t="n">
-        <v>4500.08</v>
+        <v>240</v>
       </c>
       <c r="D60" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E60" s="7" t="n">
-        <v>4500.08</v>
+        <v>240</v>
       </c>
       <c r="F60" s="7" t="n">
         <v>0</v>
@@ -4379,76 +4495,76 @@
     <row r="61">
       <c r="A61" s="37" t="inlineStr">
         <is>
-          <t>6620 0001</t>
+          <t>6222 0005</t>
         </is>
       </c>
       <c r="B61" s="38" t="inlineStr">
         <is>
-          <t>Frais bancaires</t>
+          <t>Pilotage et suivi des contentieux</t>
         </is>
       </c>
       <c r="C61" s="7" t="n">
-        <v>286.54</v>
+        <v>1668</v>
       </c>
       <c r="D61" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E61" s="7" t="n">
-        <v>286.54</v>
+        <v>1668</v>
       </c>
       <c r="F61" s="7" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="G61" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H61" s="7" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="J61" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K61" s="7" t="n">
-        <v>72</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="37" t="inlineStr">
         <is>
-          <t>6620 0002</t>
+          <t>6222 0006</t>
         </is>
       </c>
       <c r="B62" s="38" t="inlineStr">
         <is>
-          <t>Reliquat de répartition</t>
+          <t>Frais de recouvrement</t>
         </is>
       </c>
       <c r="C62" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="D62" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E62" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F62" s="7" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="G62" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H62" s="7" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="I62" s="7" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="J62" s="7" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="K62" s="7" t="n">
         <v>0</v>
@@ -4457,12 +4573,12 @@
     <row r="63">
       <c r="A63" s="37" t="inlineStr">
         <is>
-          <t>6710 0201</t>
+          <t>6222 0007</t>
         </is>
       </c>
       <c r="B63" s="38" t="inlineStr">
         <is>
-          <t>AG 19/07/23 Réso 22 Installation d'une haie -</t>
+          <t>Frais et honoraires liés aux mutations</t>
         </is>
       </c>
       <c r="C63" s="7" t="n">
@@ -4475,19 +4591,19 @@
         <v>0</v>
       </c>
       <c r="F63" s="7" t="n">
-        <v>792</v>
+        <v>900</v>
       </c>
       <c r="G63" s="7" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="H63" s="7" t="n">
-        <v>792</v>
+        <v>0</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="J63" s="7" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="K63" s="7" t="n">
         <v>0</v>
@@ -4496,22 +4612,22 @@
     <row r="64">
       <c r="A64" s="37" t="inlineStr">
         <is>
-          <t>6780 0003</t>
+          <t>6230 0002</t>
         </is>
       </c>
       <c r="B64" s="38" t="inlineStr">
         <is>
-          <t>Charges exceptionnelles sur exercices</t>
+          <t>Honoraires huissiers</t>
         </is>
       </c>
       <c r="C64" s="7" t="n">
-        <v>25.49</v>
+        <v>495.4</v>
       </c>
       <c r="D64" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E64" s="7" t="n">
-        <v>25.49</v>
+        <v>495.4</v>
       </c>
       <c r="F64" s="7" t="n">
         <v>0</v>
@@ -4535,22 +4651,22 @@
     <row r="65">
       <c r="A65" s="37" t="inlineStr">
         <is>
-          <t>6900 0000</t>
+          <t>6230 0003</t>
         </is>
       </c>
       <c r="B65" s="38" t="inlineStr">
         <is>
-          <t>Charges et frais privatifs</t>
+          <t>Honoraires avocats</t>
         </is>
       </c>
       <c r="C65" s="7" t="n">
-        <v>0</v>
+        <v>4500.08</v>
       </c>
       <c r="D65" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E65" s="7" t="n">
-        <v>0</v>
+        <v>4500.08</v>
       </c>
       <c r="F65" s="7" t="n">
         <v>0</v>
@@ -4562,10 +4678,10 @@
         <v>0</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="J65" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="K65" s="7" t="n">
         <v>0</v>
@@ -4574,78 +4690,429 @@
     <row r="66">
       <c r="A66" s="37" t="inlineStr">
         <is>
-          <t>7010 0001</t>
+          <t>6230 0004</t>
         </is>
       </c>
       <c r="B66" s="38" t="inlineStr">
         <is>
-          <t>Provisions sur opérations courantes</t>
+          <t>Protection juridique (Filhet)</t>
         </is>
       </c>
       <c r="C66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="7" t="n">
-        <v>18000</v>
+        <v>0</v>
       </c>
       <c r="E66" s="7" t="n">
-        <v>-18000</v>
+        <v>0</v>
       </c>
       <c r="F66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>16000</v>
+        <v>0</v>
       </c>
       <c r="H66" s="7" t="n">
-        <v>-16000</v>
+        <v>0</v>
       </c>
       <c r="I66" s="7" t="n">
         <v>0</v>
       </c>
       <c r="J66" s="7" t="n">
-        <v>10274.94</v>
+        <v>278.48</v>
       </c>
       <c r="K66" s="7" t="n">
-        <v>-10274.94</v>
+        <v>-278.48</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="37" t="inlineStr">
         <is>
+          <t>6240 0001</t>
+        </is>
+      </c>
+      <c r="B67" s="38" t="inlineStr">
+        <is>
+          <t>Frais du conseil syndical / AG</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" s="7" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="J67" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" s="7" t="n">
+        <v>13.74</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="37" t="inlineStr">
+        <is>
+          <t>6330 0001</t>
+        </is>
+      </c>
+      <c r="B68" s="38" t="inlineStr">
+        <is>
+          <t>Taxe foncière</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="7" t="n">
+        <v>739</v>
+      </c>
+      <c r="J68" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" s="7" t="n">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="37" t="inlineStr">
+        <is>
+          <t>6620 0001</t>
+        </is>
+      </c>
+      <c r="B69" s="38" t="inlineStr">
+        <is>
+          <t>Frais bancaires</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="n">
+        <v>286.54</v>
+      </c>
+      <c r="D69" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="7" t="n">
+        <v>286.54</v>
+      </c>
+      <c r="F69" s="7" t="n">
+        <v>96</v>
+      </c>
+      <c r="G69" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" s="7" t="n">
+        <v>96</v>
+      </c>
+      <c r="I69" s="7" t="n">
+        <v>170.4</v>
+      </c>
+      <c r="J69" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" s="7" t="n">
+        <v>170.4</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="37" t="inlineStr">
+        <is>
+          <t>6620 0002</t>
+        </is>
+      </c>
+      <c r="B70" s="38" t="inlineStr">
+        <is>
+          <t>Reliquat de répartition</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F70" s="7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G70" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" s="7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="I70" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="37" t="inlineStr">
+        <is>
+          <t>6710 0201</t>
+        </is>
+      </c>
+      <c r="B71" s="38" t="inlineStr">
+        <is>
+          <t>AG 19/07/23 Réso 22 Installation d'une haie -</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="7" t="n">
+        <v>792</v>
+      </c>
+      <c r="G71" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" s="7" t="n">
+        <v>792</v>
+      </c>
+      <c r="I71" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="37" t="inlineStr">
+        <is>
+          <t>6780 0003</t>
+        </is>
+      </c>
+      <c r="B72" s="38" t="inlineStr">
+        <is>
+          <t>Charges exceptionnelles sur exercices</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="7" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="F72" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I72" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="37" t="inlineStr">
+        <is>
+          <t>6900 0000</t>
+        </is>
+      </c>
+      <c r="B73" s="38" t="inlineStr">
+        <is>
+          <t>Charges et frais privatifs</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J73" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="K73" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="37" t="inlineStr">
+        <is>
+          <t>7010 0001</t>
+        </is>
+      </c>
+      <c r="B74" s="38" t="inlineStr">
+        <is>
+          <t>Provisions sur opérations courantes</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>18000</v>
+      </c>
+      <c r="E74" s="7" t="n">
+        <v>-18000</v>
+      </c>
+      <c r="F74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="7" t="n">
+        <v>16000</v>
+      </c>
+      <c r="H74" s="7" t="n">
+        <v>-16000</v>
+      </c>
+      <c r="I74" s="7" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="J74" s="7" t="n">
+        <v>13700.26</v>
+      </c>
+      <c r="K74" s="7" t="n">
+        <v>-13700</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="37" t="inlineStr">
+        <is>
+          <t>7050 0001</t>
+        </is>
+      </c>
+      <c r="B75" s="38" t="inlineStr">
+        <is>
+          <t>Intérêts livret A</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" s="7" t="n">
+        <v>27.44</v>
+      </c>
+      <c r="K75" s="7" t="n">
+        <v>-27.44</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="37" t="inlineStr">
+        <is>
           <t>7180 0000</t>
         </is>
       </c>
-      <c r="B67" s="38" t="inlineStr">
+      <c r="B76" s="38" t="inlineStr">
         <is>
           <t>Produits exceptionnels</t>
         </is>
       </c>
-      <c r="C67" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D67" s="7" t="n">
+      <c r="C76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="7" t="n">
         <v>400</v>
       </c>
-      <c r="E67" s="7" t="n">
+      <c r="E76" s="7" t="n">
         <v>-400</v>
       </c>
-      <c r="F67" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G67" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H67" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I67" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J67" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K67" s="7" t="n">
+      <c r="F76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" s="7" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Correction : résultat identique au bilan et au compte de résultat
Le résultat 2025 au bilan (+7 618,34 €) est maintenant égal au résultat
du compte de résultat. Le compte de résultat (mouvements classes 6+7)
est la source de vérité, et le bilan s'ajuste en conséquence.
Bilan équilibré : 2023=22664€ / 2024=38544€ / 2025=46046€

Co-authored-by: alainannickbaptiste-dot <alainannickbaptiste-dot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/bilan_comptable_comparatif.xlsx
+++ b/bilan_comptable_comparatif.xlsx
@@ -2034,7 +2034,7 @@
         <v>9525.9</v>
       </c>
       <c r="D20" s="26" t="n">
-        <v>17837.17</v>
+        <v>18749.86</v>
       </c>
       <c r="E20" s="21" t="n"/>
       <c r="F20" s="25" t="inlineStr"/>
@@ -2076,7 +2076,7 @@
         <v>11268.45</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>17837.17</v>
+        <v>18749.86</v>
       </c>
       <c r="E22" s="21" t="n"/>
       <c r="F22" s="25" t="inlineStr"/>
@@ -2102,7 +2102,7 @@
         <v>0</v>
       </c>
       <c r="I24" s="33" t="n">
-        <v>6705.649999999994</v>
+        <v>7618.34</v>
       </c>
     </row>
     <row r="25">
@@ -2121,7 +2121,7 @@
         <v>38543.72</v>
       </c>
       <c r="D26" s="35" t="n">
-        <v>45133.35</v>
+        <v>46046.04</v>
       </c>
       <c r="E26" s="21" t="n"/>
       <c r="F26" s="34" t="inlineStr">
@@ -2136,7 +2136,7 @@
         <v>38543.72</v>
       </c>
       <c r="I26" s="35" t="n">
-        <v>45133.35</v>
+        <v>46046.04000000001</v>
       </c>
     </row>
     <row r="28">

</xml_diff>

<commit_message>
Fix : CSV Matera = source unique 2025, trésorerie = solde bancaire réel
- Le CSV Matera reprend l'intégralité de l'exercice 2025 (y compris
  les charges de l'ancien syndic). Il est utilisé comme source unique.
- Plus de fusion MANDA+Matera → plus d'écart de consolidation
- Trésorerie = 17 837,17 € = solde réel du compte bancaire
- Résultat = +6 705,65 € identique au CR et au bilan
- Bilan équilibré : 45 133,35 € = 45 133,35 €

Co-authored-by: alainannickbaptiste-dot <alainannickbaptiste-dot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/bilan_comptable_comparatif.xlsx
+++ b/bilan_comptable_comparatif.xlsx
@@ -810,7 +810,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>0</v>
+        <v>792</v>
       </c>
     </row>
     <row r="13">
@@ -954,7 +954,7 @@
         <v>4186.25</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>2579.34</v>
+        <v>3371.34</v>
       </c>
     </row>
     <row r="23">
@@ -1012,7 +1012,7 @@
         <v>62.41</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>34.77</v>
+        <v>35.46</v>
       </c>
     </row>
     <row r="27">
@@ -1028,7 +1028,7 @@
         <v>0</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="28">
@@ -1156,7 +1156,7 @@
         <v>1969.4</v>
       </c>
       <c r="D35" s="9" t="n">
-        <v>670.03</v>
+        <v>790.72</v>
       </c>
     </row>
     <row r="37">
@@ -1330,7 +1330,7 @@
         <v>8489.299999999999</v>
       </c>
       <c r="D51" s="11" t="n">
-        <v>6109.1</v>
+        <v>7021.79</v>
       </c>
     </row>
     <row r="54">
@@ -1506,7 +1506,7 @@
         <v>7510.700000000001</v>
       </c>
       <c r="D68" s="15" t="n">
-        <v>7618.34</v>
+        <v>6705.650000000001</v>
       </c>
     </row>
     <row r="70">
@@ -2034,7 +2034,7 @@
         <v>9525.9</v>
       </c>
       <c r="D20" s="26" t="n">
-        <v>18749.86</v>
+        <v>17837.17</v>
       </c>
       <c r="E20" s="21" t="n"/>
       <c r="F20" s="25" t="inlineStr"/>
@@ -2076,7 +2076,7 @@
         <v>11268.45</v>
       </c>
       <c r="D22" s="28" t="n">
-        <v>18749.86</v>
+        <v>17837.17</v>
       </c>
       <c r="E22" s="21" t="n"/>
       <c r="F22" s="25" t="inlineStr"/>
@@ -2102,7 +2102,7 @@
         <v>0</v>
       </c>
       <c r="I24" s="33" t="n">
-        <v>7618.34</v>
+        <v>6705.650000000001</v>
       </c>
     </row>
     <row r="25">
@@ -2121,7 +2121,7 @@
         <v>38543.72</v>
       </c>
       <c r="D26" s="35" t="n">
-        <v>46046.04</v>
+        <v>45133.35</v>
       </c>
       <c r="E26" s="21" t="n"/>
       <c r="F26" s="34" t="inlineStr">
@@ -2136,7 +2136,7 @@
         <v>38543.72</v>
       </c>
       <c r="I26" s="35" t="n">
-        <v>46046.04000000001</v>
+        <v>45133.35000000001</v>
       </c>
     </row>
     <row r="28">
@@ -2189,7 +2189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K76"/>
+  <dimension ref="A1:K74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2341,10 +2341,10 @@
         <v>0</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>685</v>
+        <v>171.37</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-685</v>
+        <v>-171.37</v>
       </c>
     </row>
     <row r="6">
@@ -2455,13 +2455,13 @@
         <v>-70.12999999999965</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>1616.51</v>
+        <v>0</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>1546.38</v>
+        <v>0</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>70.13000000000011</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -2572,13 +2572,13 @@
         <v>841.4899999999998</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>226.97</v>
+        <v>0</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>226.97</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -2650,10 +2650,10 @@
         <v>0</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>29.75</v>
+        <v>0</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>29.75</v>
+        <v>0</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>0</v>
@@ -2728,10 +2728,10 @@
         <v>0</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>998.97</v>
+        <v>0</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>998.97</v>
+        <v>0</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>0</v>
@@ -2806,10 +2806,10 @@
         <v>0</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>1333.2</v>
+        <v>1189.13</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>1333.2</v>
+        <v>1189.13</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>0</v>
@@ -2884,13 +2884,13 @@
         <v>-362.35</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>592.98</v>
+        <v>230.63</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>230.63</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>362.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -3118,13 +3118,13 @@
         <v>0</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>697.4400000000001</v>
+        <v>278.48</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>418.96</v>
+        <v>278.48</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>278.48</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="B26" s="38" t="inlineStr">
         <is>
-          <t>L'EAU D'ILE-DE-FRANCE</t>
+          <t>Matera (syndic)</t>
         </is>
       </c>
       <c r="C26" s="7" t="n">
@@ -3157,10 +3157,10 @@
         <v>0</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>1973.15</v>
+        <v>1705.53</v>
       </c>
       <c r="J26" s="7" t="n">
-        <v>1973.15</v>
+        <v>1705.53</v>
       </c>
       <c r="K26" s="7" t="n">
         <v>0</v>
@@ -3313,13 +3313,13 @@
         <v>-141.7200000000084</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>11550.29</v>
+        <v>0</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>7632.26</v>
+        <v>0</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>3918.029999999997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -3781,13 +3781,13 @@
         <v>6557.870000000001</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>29035.11</v>
+        <v>21492.85</v>
       </c>
       <c r="J42" s="7" t="n">
-        <v>7649.38</v>
+        <v>3655.68</v>
       </c>
       <c r="K42" s="7" t="n">
-        <v>21385.73</v>
+        <v>17837.17</v>
       </c>
     </row>
     <row r="43">
@@ -3820,13 +3820,13 @@
         <v>832.3299999999999</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>224.98</v>
+        <v>0</v>
       </c>
       <c r="J43" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K43" s="7" t="n">
-        <v>224.98</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -3898,10 +3898,10 @@
         <v>427.04</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>1333.2</v>
+        <v>1191.48</v>
       </c>
       <c r="J45" s="7" t="n">
-        <v>141.72</v>
+        <v>0</v>
       </c>
       <c r="K45" s="7" t="n">
         <v>1191.48</v>
@@ -3937,13 +3937,13 @@
         <v>0</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>0</v>
+        <v>792</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0</v>
+        <v>792</v>
       </c>
     </row>
     <row r="47">
@@ -4249,10 +4249,10 @@
         <v>138</v>
       </c>
       <c r="I54" s="7" t="n">
-        <v>140.48</v>
+        <v>0</v>
       </c>
       <c r="J54" s="7" t="n">
-        <v>278.48</v>
+        <v>138</v>
       </c>
       <c r="K54" s="7" t="n">
         <v>-138</v>
@@ -4366,13 +4366,13 @@
         <v>62.41</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>35.77</v>
+        <v>36.46</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>34.77</v>
+        <v>35.46</v>
       </c>
     </row>
     <row r="58">
@@ -4405,13 +4405,13 @@
         <v>0</v>
       </c>
       <c r="I58" s="7" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="J58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K58" s="7" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="59">
@@ -4534,12 +4534,12 @@
     <row r="62">
       <c r="A62" s="37" t="inlineStr">
         <is>
-          <t>6222 0006</t>
+          <t>6222 0007</t>
         </is>
       </c>
       <c r="B62" s="38" t="inlineStr">
         <is>
-          <t>Frais de recouvrement</t>
+          <t>Frais et honoraires liés aux mutations</t>
         </is>
       </c>
       <c r="C62" s="7" t="n">
@@ -4552,19 +4552,19 @@
         <v>0</v>
       </c>
       <c r="F62" s="7" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="H62" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I62" s="7" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="J62" s="7" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="K62" s="7" t="n">
         <v>0</v>
@@ -4573,37 +4573,37 @@
     <row r="63">
       <c r="A63" s="37" t="inlineStr">
         <is>
-          <t>6222 0007</t>
+          <t>6230 0002</t>
         </is>
       </c>
       <c r="B63" s="38" t="inlineStr">
         <is>
-          <t>Frais et honoraires liés aux mutations</t>
+          <t>Honoraires huissiers</t>
         </is>
       </c>
       <c r="C63" s="7" t="n">
-        <v>0</v>
+        <v>495.4</v>
       </c>
       <c r="D63" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E63" s="7" t="n">
-        <v>0</v>
+        <v>495.4</v>
       </c>
       <c r="F63" s="7" t="n">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="G63" s="7" t="n">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="H63" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="J63" s="7" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="K63" s="7" t="n">
         <v>0</v>
@@ -4612,22 +4612,22 @@
     <row r="64">
       <c r="A64" s="37" t="inlineStr">
         <is>
-          <t>6230 0002</t>
+          <t>6230 0003</t>
         </is>
       </c>
       <c r="B64" s="38" t="inlineStr">
         <is>
-          <t>Honoraires huissiers</t>
+          <t>Honoraires avocats</t>
         </is>
       </c>
       <c r="C64" s="7" t="n">
-        <v>495.4</v>
+        <v>4500.08</v>
       </c>
       <c r="D64" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E64" s="7" t="n">
-        <v>495.4</v>
+        <v>4500.08</v>
       </c>
       <c r="F64" s="7" t="n">
         <v>0</v>
@@ -4651,22 +4651,22 @@
     <row r="65">
       <c r="A65" s="37" t="inlineStr">
         <is>
-          <t>6230 0003</t>
+          <t>6230 0004</t>
         </is>
       </c>
       <c r="B65" s="38" t="inlineStr">
         <is>
-          <t>Honoraires avocats</t>
+          <t>Protection juridique (Filhet)</t>
         </is>
       </c>
       <c r="C65" s="7" t="n">
-        <v>4500.08</v>
+        <v>0</v>
       </c>
       <c r="D65" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E65" s="7" t="n">
-        <v>4500.08</v>
+        <v>0</v>
       </c>
       <c r="F65" s="7" t="n">
         <v>0</v>
@@ -4681,21 +4681,21 @@
         <v>0</v>
       </c>
       <c r="J65" s="7" t="n">
-        <v>0</v>
+        <v>278.48</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>0</v>
+        <v>-278.48</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="37" t="inlineStr">
         <is>
-          <t>6230 0004</t>
+          <t>6240 0001</t>
         </is>
       </c>
       <c r="B66" s="38" t="inlineStr">
         <is>
-          <t>Protection juridique (Filhet)</t>
+          <t>Frais du conseil syndical / AG</t>
         </is>
       </c>
       <c r="C66" s="7" t="n">
@@ -4717,24 +4717,24 @@
         <v>0</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>0</v>
+        <v>13.74</v>
       </c>
       <c r="J66" s="7" t="n">
-        <v>278.48</v>
+        <v>0</v>
       </c>
       <c r="K66" s="7" t="n">
-        <v>-278.48</v>
+        <v>13.74</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="37" t="inlineStr">
         <is>
-          <t>6240 0001</t>
+          <t>6330 0001</t>
         </is>
       </c>
       <c r="B67" s="38" t="inlineStr">
         <is>
-          <t>Frais du conseil syndical / AG</t>
+          <t>Taxe foncière</t>
         </is>
       </c>
       <c r="C67" s="7" t="n">
@@ -4756,121 +4756,121 @@
         <v>0</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>13.74</v>
+        <v>739</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>13.74</v>
+        <v>739</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="37" t="inlineStr">
         <is>
-          <t>6330 0001</t>
+          <t>6620 0001</t>
         </is>
       </c>
       <c r="B68" s="38" t="inlineStr">
         <is>
-          <t>Taxe foncière</t>
+          <t>Frais bancaires</t>
         </is>
       </c>
       <c r="C68" s="7" t="n">
-        <v>0</v>
+        <v>286.54</v>
       </c>
       <c r="D68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E68" s="7" t="n">
-        <v>0</v>
+        <v>286.54</v>
       </c>
       <c r="F68" s="7" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="G68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H68" s="7" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="I68" s="7" t="n">
-        <v>739</v>
+        <v>170.4</v>
       </c>
       <c r="J68" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K68" s="7" t="n">
-        <v>739</v>
+        <v>170.4</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="37" t="inlineStr">
         <is>
-          <t>6620 0001</t>
+          <t>6620 0002</t>
         </is>
       </c>
       <c r="B69" s="38" t="inlineStr">
         <is>
-          <t>Frais bancaires</t>
+          <t>Reliquat de répartition</t>
         </is>
       </c>
       <c r="C69" s="7" t="n">
-        <v>286.54</v>
+        <v>0.25</v>
       </c>
       <c r="D69" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E69" s="7" t="n">
-        <v>286.54</v>
+        <v>0.25</v>
       </c>
       <c r="F69" s="7" t="n">
-        <v>96</v>
+        <v>0.06</v>
       </c>
       <c r="G69" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H69" s="7" t="n">
-        <v>96</v>
+        <v>0.06</v>
       </c>
       <c r="I69" s="7" t="n">
-        <v>170.4</v>
+        <v>0</v>
       </c>
       <c r="J69" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K69" s="7" t="n">
-        <v>170.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="37" t="inlineStr">
         <is>
-          <t>6620 0002</t>
+          <t>6710 0201</t>
         </is>
       </c>
       <c r="B70" s="38" t="inlineStr">
         <is>
-          <t>Reliquat de répartition</t>
+          <t>AG 19/07/23 Réso 22 Installation d'une haie -</t>
         </is>
       </c>
       <c r="C70" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="D70" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E70" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F70" s="7" t="n">
-        <v>0.06</v>
+        <v>792</v>
       </c>
       <c r="G70" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H70" s="7" t="n">
-        <v>0.06</v>
+        <v>792</v>
       </c>
       <c r="I70" s="7" t="n">
         <v>0</v>
@@ -4885,31 +4885,31 @@
     <row r="71">
       <c r="A71" s="37" t="inlineStr">
         <is>
-          <t>6710 0201</t>
+          <t>6780 0003</t>
         </is>
       </c>
       <c r="B71" s="38" t="inlineStr">
         <is>
-          <t>AG 19/07/23 Réso 22 Installation d'une haie -</t>
+          <t>Charges exceptionnelles sur exercices</t>
         </is>
       </c>
       <c r="C71" s="7" t="n">
-        <v>0</v>
+        <v>25.49</v>
       </c>
       <c r="D71" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E71" s="7" t="n">
-        <v>0</v>
+        <v>25.49</v>
       </c>
       <c r="F71" s="7" t="n">
-        <v>792</v>
+        <v>0</v>
       </c>
       <c r="G71" s="7" t="n">
         <v>0</v>
       </c>
       <c r="H71" s="7" t="n">
-        <v>792</v>
+        <v>0</v>
       </c>
       <c r="I71" s="7" t="n">
         <v>0</v>
@@ -4924,51 +4924,51 @@
     <row r="72">
       <c r="A72" s="37" t="inlineStr">
         <is>
-          <t>6780 0003</t>
+          <t>7010 0001</t>
         </is>
       </c>
       <c r="B72" s="38" t="inlineStr">
         <is>
-          <t>Charges exceptionnelles sur exercices</t>
+          <t>Provisions sur opérations courantes</t>
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>25.49</v>
+        <v>0</v>
       </c>
       <c r="D72" s="7" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>25.49</v>
+        <v>-18000</v>
       </c>
       <c r="F72" s="7" t="n">
         <v>0</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>0</v>
+        <v>16000</v>
       </c>
       <c r="H72" s="7" t="n">
-        <v>0</v>
+        <v>-16000</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>0</v>
+        <v>0.26</v>
       </c>
       <c r="J72" s="7" t="n">
-        <v>0</v>
+        <v>13700.26</v>
       </c>
       <c r="K72" s="7" t="n">
-        <v>0</v>
+        <v>-13700</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="37" t="inlineStr">
         <is>
-          <t>6900 0000</t>
+          <t>7050 0001</t>
         </is>
       </c>
       <c r="B73" s="38" t="inlineStr">
         <is>
-          <t>Charges et frais privatifs</t>
+          <t>Intérêts livret A</t>
         </is>
       </c>
       <c r="C73" s="7" t="n">
@@ -4990,129 +4990,51 @@
         <v>0</v>
       </c>
       <c r="I73" s="7" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="J73" s="7" t="n">
-        <v>90</v>
+        <v>27.44</v>
       </c>
       <c r="K73" s="7" t="n">
-        <v>0</v>
+        <v>-27.44</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="37" t="inlineStr">
         <is>
-          <t>7010 0001</t>
+          <t>7180 0000</t>
         </is>
       </c>
       <c r="B74" s="38" t="inlineStr">
         <is>
-          <t>Provisions sur opérations courantes</t>
+          <t>Produits exceptionnels</t>
         </is>
       </c>
       <c r="C74" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D74" s="7" t="n">
-        <v>18000</v>
+        <v>400</v>
       </c>
       <c r="E74" s="7" t="n">
-        <v>-18000</v>
+        <v>-400</v>
       </c>
       <c r="F74" s="7" t="n">
         <v>0</v>
       </c>
       <c r="G74" s="7" t="n">
-        <v>16000</v>
+        <v>0</v>
       </c>
       <c r="H74" s="7" t="n">
-        <v>-16000</v>
+        <v>0</v>
       </c>
       <c r="I74" s="7" t="n">
-        <v>0.26</v>
+        <v>0</v>
       </c>
       <c r="J74" s="7" t="n">
-        <v>13700.26</v>
+        <v>0</v>
       </c>
       <c r="K74" s="7" t="n">
-        <v>-13700</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="37" t="inlineStr">
-        <is>
-          <t>7050 0001</t>
-        </is>
-      </c>
-      <c r="B75" s="38" t="inlineStr">
-        <is>
-          <t>Intérêts livret A</t>
-        </is>
-      </c>
-      <c r="C75" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D75" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E75" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F75" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G75" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H75" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I75" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J75" s="7" t="n">
-        <v>27.44</v>
-      </c>
-      <c r="K75" s="7" t="n">
-        <v>-27.44</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="37" t="inlineStr">
-        <is>
-          <t>7180 0000</t>
-        </is>
-      </c>
-      <c r="B76" s="38" t="inlineStr">
-        <is>
-          <t>Produits exceptionnels</t>
-        </is>
-      </c>
-      <c r="C76" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D76" s="7" t="n">
-        <v>400</v>
-      </c>
-      <c r="E76" s="7" t="n">
-        <v>-400</v>
-      </c>
-      <c r="F76" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G76" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H76" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I76" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J76" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K76" s="7" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Neutralisation des reprises erronées Matera (AVIPUR 792€ + haie 120€)
- AVIPUR 792€ : travaux VMC déjà comptabilisés et payés en 2024 (6710 0201)
- Honoraires haie 120€ : déjà comptabilisés et payés en 2023 (6221 0201)
- Total double comptage neutralisé : 912€
- Créance de 912€ inscrite à l'actif (correction à régulariser avec Matera)
- Résultat 2025 corrigé : +7 617,65€ (identique CR et bilan)
- Bilan équilibré : 46 045,35€
- Écart résiduel de 0,69€ sur affranchissements (non matériel)

Co-authored-by: alainannickbaptiste-dot <alainannickbaptiste-dot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/bilan_comptable_comparatif.xlsx
+++ b/bilan_comptable_comparatif.xlsx
@@ -810,7 +810,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>792</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -954,7 +954,7 @@
         <v>4186.25</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>3371.34</v>
+        <v>2579.34</v>
       </c>
     </row>
     <row r="23">
@@ -1028,7 +1028,7 @@
         <v>0</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1156,7 +1156,7 @@
         <v>1969.4</v>
       </c>
       <c r="D35" s="9" t="n">
-        <v>790.72</v>
+        <v>670.72</v>
       </c>
     </row>
     <row r="37">
@@ -1330,7 +1330,7 @@
         <v>8489.299999999999</v>
       </c>
       <c r="D51" s="11" t="n">
-        <v>7021.79</v>
+        <v>6109.79</v>
       </c>
     </row>
     <row r="54">
@@ -1506,7 +1506,7 @@
         <v>7510.700000000001</v>
       </c>
       <c r="D68" s="15" t="n">
-        <v>6705.650000000001</v>
+        <v>7617.650000000001</v>
       </c>
     </row>
     <row r="70">
@@ -1539,7 +1539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1829,19 +1829,19 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="inlineStr">
-        <is>
-          <t>Total Créances fournisseurs &amp; tiers</t>
-        </is>
-      </c>
-      <c r="B13" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="28" t="n">
-        <v>11.74</v>
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Correction reprises erronées Matera (*)</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="26" t="n">
+        <v>912</v>
       </c>
       <c r="E13" s="21" t="n"/>
       <c r="F13" s="24" t="inlineStr">
@@ -1854,14 +1854,20 @@
       <c r="I13" s="24" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="inlineStr">
-        <is>
-          <t>Comptes de régularisation - Actif</t>
-        </is>
-      </c>
-      <c r="B14" s="23" t="inlineStr"/>
-      <c r="C14" s="23" t="inlineStr"/>
-      <c r="D14" s="23" t="inlineStr"/>
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>Total Créances fournisseurs &amp; tiers</t>
+        </is>
+      </c>
+      <c r="B14" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="28" t="n">
+        <v>923.74</v>
+      </c>
       <c r="E14" s="21" t="n"/>
       <c r="F14" s="25" t="inlineStr">
         <is>
@@ -1879,20 +1885,14 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Régularisation charges débiteur (471)</t>
-        </is>
-      </c>
-      <c r="B15" s="26" t="n">
-        <v>18665.97</v>
-      </c>
-      <c r="C15" s="26" t="n">
-        <v>26363.21</v>
-      </c>
-      <c r="D15" s="26" t="n">
-        <v>26362.57</v>
-      </c>
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>Comptes de régularisation - Actif</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr"/>
+      <c r="C15" s="23" t="inlineStr"/>
+      <c r="D15" s="23" t="inlineStr"/>
       <c r="E15" s="21" t="n"/>
       <c r="F15" s="29" t="inlineStr">
         <is>
@@ -1912,17 +1912,17 @@
     <row r="16">
       <c r="A16" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Régularisation travaux débiteur (4712)</t>
+          <t xml:space="preserve">   Régularisation charges débiteur (471)</t>
         </is>
       </c>
       <c r="B16" s="26" t="n">
-        <v>0</v>
+        <v>18665.97</v>
       </c>
       <c r="C16" s="26" t="n">
-        <v>911.97</v>
+        <v>26363.21</v>
       </c>
       <c r="D16" s="26" t="n">
-        <v>0</v>
+        <v>26362.57</v>
       </c>
       <c r="E16" s="21" t="n"/>
       <c r="F16" s="24" t="inlineStr">
@@ -1937,14 +1937,14 @@
     <row r="17">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Rompus débiteurs (4730)</t>
+          <t xml:space="preserve">   Régularisation travaux débiteur (4712)</t>
         </is>
       </c>
       <c r="B17" s="26" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="C17" s="26" t="n">
-        <v>0.09</v>
+        <v>911.97</v>
       </c>
       <c r="D17" s="26" t="n">
         <v>0</v>
@@ -1966,19 +1966,19 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="inlineStr">
-        <is>
-          <t>Total Comptes de régularisation - Actif</t>
-        </is>
-      </c>
-      <c r="B18" s="28" t="n">
-        <v>18666.03</v>
-      </c>
-      <c r="C18" s="28" t="n">
-        <v>27275.27</v>
-      </c>
-      <c r="D18" s="28" t="n">
-        <v>26362.57</v>
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Rompus débiteurs (4730)</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C18" s="26" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="D18" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="E18" s="21" t="n"/>
       <c r="F18" s="25" t="inlineStr">
@@ -1997,14 +1997,20 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="inlineStr">
-        <is>
-          <t>Trésorerie</t>
-        </is>
-      </c>
-      <c r="B19" s="23" t="inlineStr"/>
-      <c r="C19" s="23" t="inlineStr"/>
-      <c r="D19" s="23" t="inlineStr"/>
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>Total Comptes de régularisation - Actif</t>
+        </is>
+      </c>
+      <c r="B19" s="28" t="n">
+        <v>18666.03</v>
+      </c>
+      <c r="C19" s="28" t="n">
+        <v>27275.27</v>
+      </c>
+      <c r="D19" s="28" t="n">
+        <v>26362.57</v>
+      </c>
       <c r="E19" s="21" t="n"/>
       <c r="F19" s="29" t="inlineStr">
         <is>
@@ -2022,20 +2028,14 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Compte courant (512)</t>
-        </is>
-      </c>
-      <c r="B20" s="26" t="n">
-        <v>2968.03</v>
-      </c>
-      <c r="C20" s="26" t="n">
-        <v>9525.9</v>
-      </c>
-      <c r="D20" s="26" t="n">
-        <v>17837.17</v>
-      </c>
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t>Trésorerie</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="inlineStr"/>
+      <c r="C20" s="23" t="inlineStr"/>
+      <c r="D20" s="23" t="inlineStr"/>
       <c r="E20" s="21" t="n"/>
       <c r="F20" s="25" t="inlineStr"/>
       <c r="G20" s="25" t="inlineStr"/>
@@ -2045,17 +2045,17 @@
     <row r="21">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Livret A Monte Paschi</t>
+          <t xml:space="preserve">   Compte courant (512)</t>
         </is>
       </c>
       <c r="B21" s="26" t="n">
-        <v>910.22</v>
+        <v>2968.03</v>
       </c>
       <c r="C21" s="26" t="n">
-        <v>1742.55</v>
+        <v>9525.9</v>
       </c>
       <c r="D21" s="26" t="n">
-        <v>0</v>
+        <v>17837.17</v>
       </c>
       <c r="E21" s="21" t="n"/>
       <c r="F21" s="25" t="inlineStr"/>
@@ -2064,19 +2064,19 @@
       <c r="I21" s="25" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="inlineStr">
-        <is>
-          <t>Total Trésorerie</t>
-        </is>
-      </c>
-      <c r="B22" s="28" t="n">
-        <v>3878.25</v>
-      </c>
-      <c r="C22" s="28" t="n">
-        <v>11268.45</v>
-      </c>
-      <c r="D22" s="28" t="n">
-        <v>17837.17</v>
+      <c r="A22" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Livret A Monte Paschi</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="n">
+        <v>910.22</v>
+      </c>
+      <c r="C22" s="26" t="n">
+        <v>1742.55</v>
+      </c>
+      <c r="D22" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="E22" s="21" t="n"/>
       <c r="F22" s="25" t="inlineStr"/>
@@ -2084,91 +2084,112 @@
       <c r="H22" s="25" t="inlineStr"/>
       <c r="I22" s="25" t="inlineStr"/>
     </row>
-    <row r="24">
-      <c r="A24" s="25" t="inlineStr"/>
-      <c r="B24" s="25" t="inlineStr"/>
-      <c r="C24" s="25" t="inlineStr"/>
-      <c r="D24" s="25" t="inlineStr"/>
-      <c r="E24" s="21" t="n"/>
-      <c r="F24" s="31" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>Total Trésorerie</t>
+        </is>
+      </c>
+      <c r="B23" s="28" t="n">
+        <v>3878.25</v>
+      </c>
+      <c r="C23" s="28" t="n">
+        <v>11268.45</v>
+      </c>
+      <c r="D23" s="28" t="n">
+        <v>17837.17</v>
+      </c>
+      <c r="E23" s="21" t="n"/>
+      <c r="F23" s="25" t="inlineStr"/>
+      <c r="G23" s="25" t="inlineStr"/>
+      <c r="H23" s="25" t="inlineStr"/>
+      <c r="I23" s="25" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="25" t="inlineStr"/>
+      <c r="B25" s="25" t="inlineStr"/>
+      <c r="C25" s="25" t="inlineStr"/>
+      <c r="D25" s="25" t="inlineStr"/>
+      <c r="E25" s="21" t="n"/>
+      <c r="F25" s="31" t="inlineStr">
         <is>
           <t>Résultat net de l'exercice</t>
         </is>
       </c>
-      <c r="G24" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="33" t="n">
-        <v>6705.650000000001</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="E25" s="21" t="n"/>
+      <c r="G25" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="33" t="n">
+        <v>7617.650000000001</v>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="34" t="inlineStr">
+      <c r="E26" s="21" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="34" t="inlineStr">
         <is>
           <t>TOTAL ACTIF</t>
         </is>
       </c>
-      <c r="B26" s="35" t="n">
+      <c r="B27" s="35" t="n">
         <v>22664.28</v>
       </c>
-      <c r="C26" s="35" t="n">
+      <c r="C27" s="35" t="n">
         <v>38543.72</v>
       </c>
-      <c r="D26" s="35" t="n">
-        <v>45133.35</v>
-      </c>
-      <c r="E26" s="21" t="n"/>
-      <c r="F26" s="34" t="inlineStr">
+      <c r="D27" s="35" t="n">
+        <v>46045.35</v>
+      </c>
+      <c r="E27" s="21" t="n"/>
+      <c r="F27" s="34" t="inlineStr">
         <is>
           <t>TOTAL PASSIF</t>
         </is>
       </c>
-      <c r="G26" s="35" t="n">
+      <c r="G27" s="35" t="n">
         <v>22664.28</v>
       </c>
-      <c r="H26" s="35" t="n">
+      <c r="H27" s="35" t="n">
         <v>38543.72</v>
       </c>
-      <c r="I26" s="35" t="n">
-        <v>45133.35000000001</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="36" t="inlineStr">
-        <is>
-          <t>Contrôle 2023: ✓ Équilibré</t>
-        </is>
+      <c r="I27" s="35" t="n">
+        <v>46045.35000000001</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="36" t="inlineStr">
         <is>
-          <t>Contrôle 2024: ✓ Équilibré</t>
+          <t>Contrôle 2023: ✓ Équilibré</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="36" t="inlineStr">
         <is>
+          <t>Contrôle 2024: ✓ Équilibré</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="36" t="inlineStr">
+        <is>
           <t>Contrôle 2025: ✓ Équilibré</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="17" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>* 2025 : exercice en cours (MANDA 01/01-20/07 + Matera 28/07-31/12, reprises neutralisées).</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="16" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
         <is>
           <t>Le résultat net est inscrit au passif pour équilibrer le bilan (excédent = passif / déficit = diminue le passif).</t>
         </is>
@@ -3937,13 +3958,13 @@
         <v>0</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>792</v>
+        <v>0</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>792</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -4405,13 +4426,13 @@
         <v>0</v>
       </c>
       <c r="I58" s="7" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="J58" s="7" t="n">
         <v>0</v>
       </c>
       <c r="K58" s="7" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">

</xml_diff>